<commit_message>
Reescritura completa del modulo Inventario (HTML/CSS/JS limpios y funcionales)
</commit_message>
<xml_diff>
--- a/Inventario Diciembre.xlsx
+++ b/Inventario Diciembre.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anime\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b751df8fdfd3fc6f/Documentos/GitHub/willianworkshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CCFD0E0-91E2-432E-9EC5-28D300F50351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{3CCFD0E0-91E2-432E-9EC5-28D300F50351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{637AD33F-6749-437A-AA97-030EA40D7274}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{36D6B9B6-F2BD-47F5-95D5-897B11381D8C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja2" sheetId="2" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -48,9 +48,6 @@
     <t>Descripcion según factura</t>
   </si>
   <si>
-    <t>Precio costo</t>
-  </si>
-  <si>
     <t>Precio de venta</t>
   </si>
   <si>
@@ -1135,14 +1132,36 @@
   </si>
   <si>
     <t>STOCK</t>
+  </si>
+  <si>
+    <t>Precio de costo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1167,13 +1186,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1492,29 +1521,29 @@
     <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="45.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>365</v>
+      <c r="F1" s="2" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1522,12 +1551,12 @@
         <v>3401502</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1">
         <v>7</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="1">
         <v>12</v>
       </c>
       <c r="F2">
@@ -1536,15 +1565,15 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3">
+      <c r="D3" s="1">
         <v>10</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="1">
         <v>15</v>
       </c>
       <c r="F3">
@@ -1553,12 +1582,12 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4">
+      <c r="E4" s="1">
         <v>16</v>
       </c>
       <c r="F4">
@@ -1567,12 +1596,12 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5">
+      <c r="E5" s="1">
         <v>16</v>
       </c>
       <c r="F5">
@@ -1584,15 +1613,15 @@
         <v>3406</v>
       </c>
       <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
         <v>12</v>
       </c>
-      <c r="C6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6">
+      <c r="D6" s="1">
         <v>0.19209999999999999</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="1">
         <v>1</v>
       </c>
       <c r="F6">
@@ -1604,12 +1633,12 @@
         <v>52240764</v>
       </c>
       <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
         <v>14</v>
       </c>
-      <c r="C7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7">
+      <c r="E7" s="1">
         <v>20</v>
       </c>
       <c r="F7">
@@ -1621,12 +1650,12 @@
         <v>31101020</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8">
+        <v>15</v>
+      </c>
+      <c r="D8" s="1">
         <v>3.5</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="1">
         <v>7</v>
       </c>
       <c r="F8">
@@ -1635,9 +1664,9 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9">
+        <v>16</v>
+      </c>
+      <c r="E9" s="1">
         <v>3</v>
       </c>
       <c r="F9">
@@ -1646,9 +1675,9 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>18</v>
-      </c>
-      <c r="E10">
+        <v>17</v>
+      </c>
+      <c r="E10" s="1">
         <v>2</v>
       </c>
       <c r="F10">
@@ -1657,9 +1686,9 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11">
+        <v>18</v>
+      </c>
+      <c r="E11" s="1">
         <v>6</v>
       </c>
       <c r="F11">
@@ -1668,9 +1697,9 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12">
+        <v>19</v>
+      </c>
+      <c r="E12" s="1">
         <v>7</v>
       </c>
       <c r="F12">
@@ -1682,15 +1711,15 @@
         <v>39143520</v>
       </c>
       <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s">
         <v>21</v>
       </c>
-      <c r="C13" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13">
+      <c r="D13" s="1">
         <v>1.699972</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="1">
         <v>5</v>
       </c>
       <c r="F13">
@@ -1699,9 +1728,9 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
-        <v>23</v>
-      </c>
-      <c r="E14">
+        <v>22</v>
+      </c>
+      <c r="E14" s="1">
         <v>8</v>
       </c>
       <c r="F14">
@@ -1710,9 +1739,9 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E15">
+        <v>23</v>
+      </c>
+      <c r="E15" s="1">
         <v>13.5</v>
       </c>
       <c r="F15">
@@ -1721,9 +1750,9 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
-        <v>25</v>
-      </c>
-      <c r="E16">
+        <v>24</v>
+      </c>
+      <c r="E16" s="1">
         <v>5</v>
       </c>
       <c r="F16">
@@ -1732,18 +1761,18 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" t="s">
         <v>26</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>27</v>
       </c>
-      <c r="C17" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17">
+      <c r="D17" s="1">
         <v>1.0508999999999999</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="1">
         <v>3</v>
       </c>
       <c r="F17">
@@ -1752,18 +1781,18 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" t="s">
         <v>29</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>30</v>
       </c>
-      <c r="C18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18">
+      <c r="D18" s="1">
         <v>1.0508999999999999</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="1">
         <v>3</v>
       </c>
       <c r="F18">
@@ -1772,18 +1801,18 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" t="s">
         <v>32</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>33</v>
       </c>
-      <c r="C19" t="s">
-        <v>34</v>
-      </c>
-      <c r="D19">
+      <c r="D19" s="1">
         <v>1.85</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="1">
         <v>4</v>
       </c>
       <c r="F19">
@@ -1792,12 +1821,12 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" t="s">
         <v>35</v>
       </c>
-      <c r="B20" t="s">
-        <v>36</v>
-      </c>
-      <c r="E20">
+      <c r="E20" s="1">
         <v>13.5</v>
       </c>
       <c r="F20">
@@ -1806,12 +1835,12 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" t="s">
         <v>37</v>
       </c>
-      <c r="C21" t="s">
-        <v>38</v>
-      </c>
-      <c r="E21">
+      <c r="E21" s="1">
         <v>3</v>
       </c>
       <c r="F21">
@@ -1819,19 +1848,19 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22">
+      <c r="A22" s="4">
         <v>482680181601</v>
       </c>
       <c r="B22" t="s">
+        <v>38</v>
+      </c>
+      <c r="C22" t="s">
         <v>39</v>
       </c>
-      <c r="C22" t="s">
-        <v>40</v>
-      </c>
-      <c r="D22">
+      <c r="D22" s="1">
         <v>0.23119799999999999</v>
       </c>
-      <c r="E22">
+      <c r="E22" s="1">
         <v>0.5</v>
       </c>
       <c r="F22">
@@ -1840,15 +1869,15 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" t="s">
         <v>41</v>
       </c>
-      <c r="B23" t="s">
-        <v>42</v>
-      </c>
-      <c r="D23">
+      <c r="D23" s="1">
         <v>23</v>
       </c>
-      <c r="E23">
+      <c r="E23" s="1">
         <v>30</v>
       </c>
       <c r="F23">
@@ -1857,18 +1886,18 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" t="s">
         <v>43</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>44</v>
       </c>
-      <c r="C24" t="s">
-        <v>45</v>
-      </c>
-      <c r="D24">
+      <c r="D24" s="1">
         <v>16.995200000000001</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="1">
         <v>40</v>
       </c>
       <c r="F24">
@@ -1877,15 +1906,15 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" t="s">
         <v>46</v>
       </c>
-      <c r="B25" t="s">
-        <v>47</v>
-      </c>
-      <c r="D25">
+      <c r="D25" s="1">
         <v>4.5</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="1">
         <v>7</v>
       </c>
       <c r="F25">
@@ -1894,15 +1923,15 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" t="s">
         <v>48</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>49</v>
       </c>
-      <c r="C26" t="s">
-        <v>50</v>
-      </c>
-      <c r="E26">
+      <c r="E26" s="1">
         <v>11.5</v>
       </c>
       <c r="F26">
@@ -1911,15 +1940,15 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
+        <v>50</v>
+      </c>
+      <c r="B27" t="s">
         <v>51</v>
       </c>
-      <c r="B27" t="s">
-        <v>52</v>
-      </c>
-      <c r="D27">
+      <c r="D27" s="1">
         <v>2.5</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="1">
         <v>6.5</v>
       </c>
       <c r="F27">
@@ -1928,18 +1957,18 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" t="s">
         <v>53</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>54</v>
       </c>
-      <c r="C28" t="s">
-        <v>55</v>
-      </c>
-      <c r="D28">
+      <c r="D28" s="1">
         <v>2.75</v>
       </c>
-      <c r="E28">
+      <c r="E28" s="1">
         <v>4.5</v>
       </c>
       <c r="F28">
@@ -1948,18 +1977,18 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" t="s">
         <v>56</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>57</v>
       </c>
-      <c r="C29" t="s">
-        <v>58</v>
-      </c>
-      <c r="D29">
+      <c r="D29" s="1">
         <v>1</v>
       </c>
-      <c r="E29">
+      <c r="E29" s="1">
         <v>3</v>
       </c>
       <c r="F29">
@@ -1968,15 +1997,15 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" t="s">
         <v>59</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>60</v>
       </c>
-      <c r="C30" t="s">
-        <v>61</v>
-      </c>
-      <c r="E30">
+      <c r="E30" s="1">
         <v>5.5</v>
       </c>
       <c r="F30">
@@ -1985,15 +2014,15 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" t="s">
         <v>62</v>
       </c>
-      <c r="B31" t="s">
-        <v>63</v>
-      </c>
-      <c r="D31">
+      <c r="D31" s="1">
         <v>16</v>
       </c>
-      <c r="E31">
+      <c r="E31" s="1">
         <v>27</v>
       </c>
       <c r="F31">
@@ -2002,15 +2031,15 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="B32" t="s">
-        <v>65</v>
-      </c>
-      <c r="D32">
+      <c r="D32" s="1">
         <v>9</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="1">
         <v>15</v>
       </c>
       <c r="F32">
@@ -2019,15 +2048,15 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>65</v>
+      </c>
+      <c r="B33" t="s">
         <v>66</v>
       </c>
-      <c r="B33" t="s">
-        <v>67</v>
-      </c>
-      <c r="D33">
+      <c r="D33" s="1">
         <v>5</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="1">
         <v>10</v>
       </c>
       <c r="F33">
@@ -2036,15 +2065,15 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>67</v>
+      </c>
+      <c r="B34" t="s">
         <v>68</v>
       </c>
-      <c r="B34" t="s">
-        <v>69</v>
-      </c>
-      <c r="D34">
+      <c r="D34" s="1">
         <v>4</v>
       </c>
-      <c r="E34">
+      <c r="E34" s="1">
         <v>10</v>
       </c>
       <c r="F34">
@@ -2053,15 +2082,15 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>69</v>
+      </c>
+      <c r="B35" t="s">
         <v>70</v>
       </c>
-      <c r="B35" t="s">
-        <v>71</v>
-      </c>
-      <c r="D35">
+      <c r="D35" s="1">
         <v>3.25</v>
       </c>
-      <c r="E35">
+      <c r="E35" s="1">
         <v>6</v>
       </c>
       <c r="F35">
@@ -2070,18 +2099,18 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>71</v>
+      </c>
+      <c r="B36" t="s">
         <v>72</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>73</v>
       </c>
-      <c r="C36" t="s">
-        <v>74</v>
-      </c>
-      <c r="D36">
+      <c r="D36" s="1">
         <v>6</v>
       </c>
-      <c r="E36">
+      <c r="E36" s="1">
         <v>10</v>
       </c>
       <c r="F36">
@@ -2090,15 +2119,15 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
+        <v>74</v>
+      </c>
+      <c r="B37" t="s">
         <v>75</v>
       </c>
-      <c r="B37" t="s">
-        <v>76</v>
-      </c>
-      <c r="D37">
+      <c r="D37" s="1">
         <v>4</v>
       </c>
-      <c r="E37">
+      <c r="E37" s="1">
         <v>6</v>
       </c>
       <c r="F37">
@@ -2107,15 +2136,15 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
+        <v>76</v>
+      </c>
+      <c r="B38" t="s">
         <v>77</v>
       </c>
-      <c r="B38" t="s">
-        <v>78</v>
-      </c>
-      <c r="D38">
+      <c r="D38" s="1">
         <v>3.25</v>
       </c>
-      <c r="E38">
+      <c r="E38" s="1">
         <v>5.5</v>
       </c>
       <c r="F38">
@@ -2124,18 +2153,18 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" t="s">
         <v>79</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>80</v>
       </c>
-      <c r="C39" t="s">
-        <v>81</v>
-      </c>
-      <c r="D39">
+      <c r="D39" s="1">
         <v>2.5990000000000002</v>
       </c>
-      <c r="E39">
+      <c r="E39" s="1">
         <v>5</v>
       </c>
       <c r="F39">
@@ -2144,12 +2173,12 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>81</v>
+      </c>
+      <c r="B40" t="s">
         <v>82</v>
       </c>
-      <c r="B40" t="s">
-        <v>83</v>
-      </c>
-      <c r="E40">
+      <c r="E40" s="1">
         <v>10</v>
       </c>
       <c r="F40">
@@ -2158,12 +2187,12 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
+        <v>83</v>
+      </c>
+      <c r="B41" t="s">
         <v>84</v>
       </c>
-      <c r="B41" t="s">
-        <v>85</v>
-      </c>
-      <c r="E41">
+      <c r="E41" s="1">
         <v>10</v>
       </c>
       <c r="F41">
@@ -2172,9 +2201,9 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
-        <v>86</v>
-      </c>
-      <c r="E42">
+        <v>85</v>
+      </c>
+      <c r="E42" s="1">
         <v>1.5</v>
       </c>
       <c r="F42">
@@ -2183,9 +2212,9 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
-        <v>87</v>
-      </c>
-      <c r="E43">
+        <v>86</v>
+      </c>
+      <c r="E43" s="1">
         <v>1.5</v>
       </c>
       <c r="F43">
@@ -2194,12 +2223,12 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
+        <v>87</v>
+      </c>
+      <c r="C44" t="s">
         <v>88</v>
       </c>
-      <c r="C44" t="s">
-        <v>89</v>
-      </c>
-      <c r="E44">
+      <c r="E44" s="1">
         <v>7</v>
       </c>
       <c r="F44">
@@ -2208,18 +2237,18 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
+        <v>89</v>
+      </c>
+      <c r="B45" t="s">
         <v>90</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
         <v>91</v>
       </c>
-      <c r="C45" t="s">
-        <v>92</v>
-      </c>
-      <c r="D45">
+      <c r="D45" s="1">
         <v>2.4</v>
       </c>
-      <c r="E45">
+      <c r="E45" s="1">
         <v>4</v>
       </c>
       <c r="F45">
@@ -2228,15 +2257,15 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
+        <v>92</v>
+      </c>
+      <c r="B46" t="s">
         <v>93</v>
       </c>
-      <c r="B46" t="s">
-        <v>94</v>
-      </c>
-      <c r="D46">
+      <c r="D46" s="1">
         <v>1.2656000000000001</v>
       </c>
-      <c r="E46">
+      <c r="E46" s="1">
         <v>4</v>
       </c>
       <c r="F46">
@@ -2245,18 +2274,18 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
+        <v>94</v>
+      </c>
+      <c r="B47" t="s">
         <v>95</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
         <v>96</v>
       </c>
-      <c r="C47" t="s">
-        <v>97</v>
-      </c>
-      <c r="D47">
+      <c r="D47" s="1">
         <v>1.72</v>
       </c>
-      <c r="E47">
+      <c r="E47" s="1">
         <v>4.5</v>
       </c>
       <c r="F47">
@@ -2265,18 +2294,18 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
+        <v>97</v>
+      </c>
+      <c r="B48" t="s">
         <v>98</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" t="s">
         <v>99</v>
       </c>
-      <c r="C48" t="s">
-        <v>100</v>
-      </c>
-      <c r="D48">
+      <c r="D48" s="1">
         <v>2.12</v>
       </c>
-      <c r="E48">
+      <c r="E48" s="1">
         <v>4.5</v>
       </c>
       <c r="F48">
@@ -2285,15 +2314,15 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
+        <v>100</v>
+      </c>
+      <c r="B49" t="s">
         <v>101</v>
       </c>
-      <c r="B49" t="s">
-        <v>102</v>
-      </c>
-      <c r="D49">
+      <c r="D49" s="1">
         <v>43</v>
       </c>
-      <c r="E49">
+      <c r="E49" s="1">
         <v>60</v>
       </c>
       <c r="F49">
@@ -2302,15 +2331,15 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
+        <v>102</v>
+      </c>
+      <c r="B50" t="s">
         <v>103</v>
       </c>
-      <c r="B50" t="s">
-        <v>104</v>
-      </c>
-      <c r="D50">
+      <c r="D50" s="1">
         <v>33</v>
       </c>
-      <c r="E50">
+      <c r="E50" s="1">
         <v>55</v>
       </c>
       <c r="F50">
@@ -2319,12 +2348,12 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
+        <v>104</v>
+      </c>
+      <c r="B51" t="s">
         <v>105</v>
       </c>
-      <c r="B51" t="s">
-        <v>106</v>
-      </c>
-      <c r="E51">
+      <c r="E51" s="1">
         <v>40</v>
       </c>
       <c r="F51">
@@ -2333,18 +2362,18 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
+        <v>106</v>
+      </c>
+      <c r="B52" t="s">
         <v>107</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
         <v>108</v>
       </c>
-      <c r="C52" t="s">
-        <v>109</v>
-      </c>
-      <c r="D52">
+      <c r="D52" s="1">
         <v>3.75</v>
       </c>
-      <c r="E52">
+      <c r="E52" s="1">
         <v>6.5</v>
       </c>
       <c r="F52">
@@ -2356,15 +2385,15 @@
         <v>4841</v>
       </c>
       <c r="B53" t="s">
+        <v>109</v>
+      </c>
+      <c r="C53" t="s">
         <v>110</v>
       </c>
-      <c r="C53" t="s">
-        <v>111</v>
-      </c>
-      <c r="D53">
+      <c r="D53" s="1">
         <v>80.998400000000004</v>
       </c>
-      <c r="E53">
+      <c r="E53" s="1">
         <v>96</v>
       </c>
       <c r="F53">
@@ -2373,15 +2402,15 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
+        <v>111</v>
+      </c>
+      <c r="B54" t="s">
         <v>112</v>
       </c>
-      <c r="B54" t="s">
-        <v>113</v>
-      </c>
-      <c r="D54">
+      <c r="D54" s="1">
         <v>11</v>
       </c>
-      <c r="E54">
+      <c r="E54" s="1">
         <v>17</v>
       </c>
       <c r="F54">
@@ -2390,9 +2419,9 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
-        <v>114</v>
-      </c>
-      <c r="E55">
+        <v>113</v>
+      </c>
+      <c r="E55" s="1">
         <v>24.5</v>
       </c>
       <c r="F55">
@@ -2401,12 +2430,12 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
+        <v>114</v>
+      </c>
+      <c r="B56" t="s">
         <v>115</v>
       </c>
-      <c r="B56" t="s">
-        <v>116</v>
-      </c>
-      <c r="E56">
+      <c r="E56" s="1">
         <v>67</v>
       </c>
       <c r="F56">
@@ -2415,12 +2444,12 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
+        <v>116</v>
+      </c>
+      <c r="B57" t="s">
         <v>117</v>
       </c>
-      <c r="B57" t="s">
-        <v>118</v>
-      </c>
-      <c r="E57">
+      <c r="E57" s="1">
         <v>52</v>
       </c>
       <c r="F57">
@@ -2432,12 +2461,12 @@
         <v>1650101601</v>
       </c>
       <c r="B58" t="s">
+        <v>118</v>
+      </c>
+      <c r="C58" t="s">
         <v>119</v>
       </c>
-      <c r="C58" t="s">
-        <v>120</v>
-      </c>
-      <c r="E58">
+      <c r="E58" s="1">
         <v>55</v>
       </c>
       <c r="F58">
@@ -2449,12 +2478,12 @@
         <v>242477</v>
       </c>
       <c r="B59" t="s">
+        <v>120</v>
+      </c>
+      <c r="C59" t="s">
         <v>121</v>
       </c>
-      <c r="C59" t="s">
-        <v>122</v>
-      </c>
-      <c r="E59">
+      <c r="E59" s="1">
         <v>5.5</v>
       </c>
       <c r="F59">
@@ -2463,18 +2492,18 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
+        <v>122</v>
+      </c>
+      <c r="B60" t="s">
         <v>123</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C60" t="s">
         <v>124</v>
       </c>
-      <c r="C60" t="s">
-        <v>125</v>
-      </c>
-      <c r="D60">
+      <c r="D60" s="1">
         <v>7</v>
       </c>
-      <c r="E60">
+      <c r="E60" s="1">
         <v>11.5</v>
       </c>
       <c r="F60">
@@ -2483,15 +2512,15 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
+        <v>125</v>
+      </c>
+      <c r="B61" t="s">
         <v>126</v>
       </c>
-      <c r="B61" t="s">
+      <c r="C61" t="s">
         <v>127</v>
       </c>
-      <c r="C61" t="s">
-        <v>128</v>
-      </c>
-      <c r="E61">
+      <c r="E61" s="1">
         <v>11.5</v>
       </c>
       <c r="F61">
@@ -2500,18 +2529,18 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
+        <v>128</v>
+      </c>
+      <c r="B62" t="s">
         <v>129</v>
       </c>
-      <c r="B62" t="s">
+      <c r="C62" t="s">
         <v>130</v>
       </c>
-      <c r="C62" t="s">
-        <v>131</v>
-      </c>
-      <c r="D62">
+      <c r="D62" s="1">
         <v>7</v>
       </c>
-      <c r="E62">
+      <c r="E62" s="1">
         <v>11.5</v>
       </c>
       <c r="F62">
@@ -2520,12 +2549,12 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
+        <v>131</v>
+      </c>
+      <c r="B63" t="s">
         <v>132</v>
       </c>
-      <c r="B63" t="s">
-        <v>133</v>
-      </c>
-      <c r="E63">
+      <c r="E63" s="1">
         <v>32</v>
       </c>
       <c r="F63">
@@ -2534,15 +2563,15 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
+        <v>133</v>
+      </c>
+      <c r="B64" t="s">
         <v>134</v>
       </c>
-      <c r="B64" t="s">
-        <v>135</v>
-      </c>
-      <c r="D64">
+      <c r="D64" s="1">
         <v>3.75</v>
       </c>
-      <c r="E64">
+      <c r="E64" s="1">
         <v>8</v>
       </c>
       <c r="F64">
@@ -2551,15 +2580,15 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
+        <v>135</v>
+      </c>
+      <c r="B65" t="s">
         <v>136</v>
       </c>
-      <c r="B65" t="s">
-        <v>137</v>
-      </c>
-      <c r="D65">
+      <c r="D65" s="1">
         <v>60</v>
       </c>
-      <c r="E65">
+      <c r="E65" s="1">
         <v>70</v>
       </c>
       <c r="F65">
@@ -2568,15 +2597,15 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
+        <v>137</v>
+      </c>
+      <c r="B66" t="s">
         <v>138</v>
       </c>
-      <c r="B66" t="s">
-        <v>139</v>
-      </c>
-      <c r="D66">
+      <c r="D66" s="1">
         <v>8</v>
       </c>
-      <c r="E66">
+      <c r="E66" s="1">
         <v>12</v>
       </c>
       <c r="F66">
@@ -2585,15 +2614,15 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
+        <v>139</v>
+      </c>
+      <c r="B67" t="s">
         <v>140</v>
       </c>
-      <c r="B67" t="s">
-        <v>141</v>
-      </c>
-      <c r="D67">
+      <c r="D67" s="1">
         <v>10</v>
       </c>
-      <c r="E67">
+      <c r="E67" s="1">
         <v>14.5</v>
       </c>
       <c r="F67">
@@ -2602,18 +2631,18 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
+        <v>141</v>
+      </c>
+      <c r="B68" t="s">
         <v>142</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" t="s">
         <v>143</v>
       </c>
-      <c r="C68" t="s">
-        <v>144</v>
-      </c>
-      <c r="D68">
+      <c r="D68" s="1">
         <v>14</v>
       </c>
-      <c r="E68">
+      <c r="E68" s="1">
         <v>23</v>
       </c>
       <c r="F68">
@@ -2622,15 +2651,15 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
+        <v>144</v>
+      </c>
+      <c r="B69" t="s">
         <v>145</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C69" t="s">
         <v>146</v>
       </c>
-      <c r="C69" t="s">
-        <v>147</v>
-      </c>
-      <c r="E69">
+      <c r="E69" s="1">
         <v>17.5</v>
       </c>
       <c r="F69">
@@ -2639,12 +2668,12 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
-        <v>148</v>
-      </c>
-      <c r="D70">
+        <v>147</v>
+      </c>
+      <c r="D70" s="1">
         <v>10.531599999999999</v>
       </c>
-      <c r="E70">
+      <c r="E70" s="1">
         <v>20</v>
       </c>
       <c r="F70">
@@ -2653,18 +2682,18 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
+        <v>148</v>
+      </c>
+      <c r="B71" t="s">
         <v>149</v>
       </c>
-      <c r="B71" t="s">
+      <c r="C71" t="s">
         <v>150</v>
       </c>
-      <c r="C71" t="s">
-        <v>151</v>
-      </c>
-      <c r="D71">
+      <c r="D71" s="1">
         <v>0.4</v>
       </c>
-      <c r="E71">
+      <c r="E71" s="1">
         <v>1.5</v>
       </c>
       <c r="F71">
@@ -2676,9 +2705,9 @@
         <v>2871</v>
       </c>
       <c r="B72" t="s">
-        <v>152</v>
-      </c>
-      <c r="E72">
+        <v>151</v>
+      </c>
+      <c r="E72" s="1">
         <v>3</v>
       </c>
       <c r="F72">
@@ -2687,18 +2716,18 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
+        <v>152</v>
+      </c>
+      <c r="B73" t="s">
         <v>153</v>
       </c>
-      <c r="B73" t="s">
+      <c r="C73" t="s">
         <v>154</v>
       </c>
-      <c r="C73" t="s">
-        <v>155</v>
-      </c>
-      <c r="D73">
+      <c r="D73" s="1">
         <v>2</v>
       </c>
-      <c r="E73">
+      <c r="E73" s="1">
         <v>3.5</v>
       </c>
       <c r="F73">
@@ -2707,15 +2736,15 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
+        <v>155</v>
+      </c>
+      <c r="B74" t="s">
         <v>156</v>
       </c>
-      <c r="B74" t="s">
+      <c r="C74" t="s">
         <v>157</v>
       </c>
-      <c r="C74" t="s">
-        <v>158</v>
-      </c>
-      <c r="E74">
+      <c r="E74" s="1">
         <v>4</v>
       </c>
       <c r="F74">
@@ -2727,9 +2756,9 @@
         <v>4092</v>
       </c>
       <c r="B75" t="s">
-        <v>159</v>
-      </c>
-      <c r="E75">
+        <v>158</v>
+      </c>
+      <c r="E75" s="1">
         <v>3</v>
       </c>
       <c r="F75">
@@ -2738,18 +2767,18 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
+        <v>159</v>
+      </c>
+      <c r="B76" t="s">
         <v>160</v>
       </c>
-      <c r="B76" t="s">
+      <c r="C76" t="s">
         <v>161</v>
       </c>
-      <c r="C76" t="s">
-        <v>162</v>
-      </c>
-      <c r="D76">
+      <c r="D76" s="1">
         <v>4</v>
       </c>
-      <c r="E76">
+      <c r="E76" s="1">
         <v>6.5</v>
       </c>
       <c r="F76">
@@ -2761,12 +2790,12 @@
         <v>28101110</v>
       </c>
       <c r="B77" t="s">
+        <v>162</v>
+      </c>
+      <c r="C77" t="s">
         <v>163</v>
       </c>
-      <c r="C77" t="s">
-        <v>164</v>
-      </c>
-      <c r="E77">
+      <c r="E77" s="1">
         <v>2</v>
       </c>
       <c r="F77">
@@ -2775,12 +2804,12 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
+        <v>164</v>
+      </c>
+      <c r="C78" t="s">
         <v>165</v>
       </c>
-      <c r="C78" t="s">
-        <v>166</v>
-      </c>
-      <c r="E78">
+      <c r="E78" s="1">
         <v>8</v>
       </c>
       <c r="F78">
@@ -2789,15 +2818,15 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
+        <v>166</v>
+      </c>
+      <c r="B79" t="s">
         <v>167</v>
       </c>
-      <c r="B79" t="s">
-        <v>168</v>
-      </c>
-      <c r="D79">
+      <c r="D79" s="1">
         <v>13</v>
       </c>
-      <c r="E79">
+      <c r="E79" s="1">
         <v>25</v>
       </c>
       <c r="F79">
@@ -2806,18 +2835,18 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
+        <v>168</v>
+      </c>
+      <c r="B80" t="s">
         <v>169</v>
       </c>
-      <c r="B80" t="s">
+      <c r="C80" t="s">
         <v>170</v>
       </c>
-      <c r="C80" t="s">
-        <v>171</v>
-      </c>
-      <c r="D80">
+      <c r="D80" s="1">
         <v>1.8532</v>
       </c>
-      <c r="E80">
+      <c r="E80" s="1">
         <v>5</v>
       </c>
       <c r="F80">
@@ -2826,18 +2855,18 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
+        <v>171</v>
+      </c>
+      <c r="B81" t="s">
         <v>172</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C81" t="s">
         <v>173</v>
       </c>
-      <c r="C81" t="s">
-        <v>174</v>
-      </c>
-      <c r="D81">
+      <c r="D81" s="1">
         <v>3.75</v>
       </c>
-      <c r="E81">
+      <c r="E81" s="1">
         <v>7</v>
       </c>
       <c r="F81">
@@ -2846,18 +2875,18 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
+        <v>174</v>
+      </c>
+      <c r="B82" t="s">
         <v>175</v>
       </c>
-      <c r="B82" t="s">
+      <c r="C82" t="s">
         <v>176</v>
       </c>
-      <c r="C82" t="s">
-        <v>177</v>
-      </c>
-      <c r="D82">
+      <c r="D82" s="1">
         <v>0.38419999999999999</v>
       </c>
-      <c r="E82">
+      <c r="E82" s="1">
         <v>1</v>
       </c>
       <c r="F82">
@@ -2866,18 +2895,18 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
+        <v>177</v>
+      </c>
+      <c r="B83" t="s">
         <v>178</v>
       </c>
-      <c r="B83" t="s">
+      <c r="C83" t="s">
         <v>179</v>
       </c>
-      <c r="C83" t="s">
-        <v>180</v>
-      </c>
-      <c r="D83">
+      <c r="D83" s="1">
         <v>10</v>
       </c>
-      <c r="E83">
+      <c r="E83" s="1">
         <v>15</v>
       </c>
       <c r="F83">
@@ -2886,18 +2915,18 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
+        <v>180</v>
+      </c>
+      <c r="B84" t="s">
         <v>181</v>
       </c>
-      <c r="B84" t="s">
+      <c r="C84" t="s">
         <v>182</v>
       </c>
-      <c r="C84" t="s">
-        <v>183</v>
-      </c>
-      <c r="D84">
+      <c r="D84" s="1">
         <v>10</v>
       </c>
-      <c r="E84">
+      <c r="E84" s="1">
         <v>15</v>
       </c>
       <c r="F84">
@@ -2909,12 +2938,12 @@
         <v>6358129273</v>
       </c>
       <c r="B85" t="s">
-        <v>184</v>
-      </c>
-      <c r="D85">
+        <v>183</v>
+      </c>
+      <c r="D85" s="1">
         <v>9.3225000000000002E-2</v>
       </c>
-      <c r="E85">
+      <c r="E85" s="1">
         <v>0.25</v>
       </c>
       <c r="F85">
@@ -2926,12 +2955,12 @@
         <v>6358129313</v>
       </c>
       <c r="B86" t="s">
-        <v>185</v>
-      </c>
-      <c r="D86">
+        <v>184</v>
+      </c>
+      <c r="D86" s="1">
         <v>9.3225000000000002E-2</v>
       </c>
-      <c r="E86">
+      <c r="E86" s="1">
         <v>0.25</v>
       </c>
       <c r="F86">
@@ -2940,15 +2969,15 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
+        <v>185</v>
+      </c>
+      <c r="B87" t="s">
         <v>186</v>
       </c>
-      <c r="B87" t="s">
-        <v>187</v>
-      </c>
-      <c r="D87">
+      <c r="D87" s="1">
         <v>0.5</v>
       </c>
-      <c r="E87">
+      <c r="E87" s="1">
         <v>1.5</v>
       </c>
       <c r="F87">
@@ -2960,15 +2989,15 @@
         <v>52244040</v>
       </c>
       <c r="B88" t="s">
+        <v>187</v>
+      </c>
+      <c r="C88" t="s">
         <v>188</v>
       </c>
-      <c r="C88" t="s">
-        <v>189</v>
-      </c>
-      <c r="D88">
+      <c r="D88" s="1">
         <v>15</v>
       </c>
-      <c r="E88">
+      <c r="E88" s="1">
         <v>20</v>
       </c>
       <c r="F88">
@@ -2980,9 +3009,9 @@
         <v>52210040</v>
       </c>
       <c r="B89" t="s">
-        <v>190</v>
-      </c>
-      <c r="E89">
+        <v>189</v>
+      </c>
+      <c r="E89" s="1">
         <v>11</v>
       </c>
       <c r="F89">
@@ -2991,18 +3020,18 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
+        <v>190</v>
+      </c>
+      <c r="B90" t="s">
         <v>191</v>
       </c>
-      <c r="B90" t="s">
+      <c r="C90" t="s">
         <v>192</v>
       </c>
-      <c r="C90" t="s">
-        <v>193</v>
-      </c>
-      <c r="D90">
+      <c r="D90" s="1">
         <v>2</v>
       </c>
-      <c r="E90">
+      <c r="E90" s="1">
         <v>3.5</v>
       </c>
       <c r="F90">
@@ -3011,18 +3040,18 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
+        <v>193</v>
+      </c>
+      <c r="B91" t="s">
         <v>194</v>
       </c>
-      <c r="B91" t="s">
+      <c r="C91" t="s">
         <v>195</v>
       </c>
-      <c r="C91" t="s">
-        <v>196</v>
-      </c>
-      <c r="D91">
+      <c r="D91" s="1">
         <v>2.5</v>
       </c>
-      <c r="E91">
+      <c r="E91" s="1">
         <v>11</v>
       </c>
       <c r="F91">
@@ -3031,12 +3060,12 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
+        <v>196</v>
+      </c>
+      <c r="B92" t="s">
         <v>197</v>
       </c>
-      <c r="B92" t="s">
-        <v>198</v>
-      </c>
-      <c r="E92">
+      <c r="E92" s="1">
         <v>6</v>
       </c>
       <c r="F92">
@@ -3045,15 +3074,15 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
+        <v>198</v>
+      </c>
+      <c r="B93" t="s">
         <v>199</v>
       </c>
-      <c r="B93" t="s">
-        <v>200</v>
-      </c>
-      <c r="D93">
+      <c r="D93" s="1">
         <v>2.5</v>
       </c>
-      <c r="E93">
+      <c r="E93" s="1">
         <v>4</v>
       </c>
       <c r="F93">
@@ -3062,15 +3091,15 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
+        <v>200</v>
+      </c>
+      <c r="B94" t="s">
         <v>201</v>
       </c>
-      <c r="B94" t="s">
-        <v>202</v>
-      </c>
-      <c r="D94">
+      <c r="D94" s="1">
         <v>6.5</v>
       </c>
-      <c r="E94">
+      <c r="E94" s="1">
         <v>12</v>
       </c>
       <c r="F94">
@@ -3079,18 +3108,18 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
+        <v>202</v>
+      </c>
+      <c r="B95" t="s">
         <v>203</v>
       </c>
-      <c r="B95" t="s">
+      <c r="C95" t="s">
         <v>204</v>
       </c>
-      <c r="C95" t="s">
-        <v>205</v>
-      </c>
-      <c r="D95">
+      <c r="D95" s="1">
         <v>6.9494999999999996</v>
       </c>
-      <c r="E95">
+      <c r="E95" s="1">
         <v>12</v>
       </c>
       <c r="F95">
@@ -3099,15 +3128,15 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
+        <v>205</v>
+      </c>
+      <c r="B96" t="s">
         <v>206</v>
       </c>
-      <c r="B96" t="s">
-        <v>207</v>
-      </c>
-      <c r="D96">
+      <c r="D96" s="1">
         <v>12.5</v>
       </c>
-      <c r="E96">
+      <c r="E96" s="1">
         <v>17</v>
       </c>
       <c r="F96">
@@ -3116,15 +3145,15 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
+        <v>207</v>
+      </c>
+      <c r="B97" t="s">
         <v>208</v>
       </c>
-      <c r="B97" t="s">
-        <v>209</v>
-      </c>
-      <c r="D97">
+      <c r="D97" s="1">
         <v>0.90400000000000003</v>
       </c>
-      <c r="E97">
+      <c r="E97" s="1">
         <v>4</v>
       </c>
       <c r="F97">
@@ -3136,9 +3165,9 @@
         <v>4092</v>
       </c>
       <c r="B98" t="s">
-        <v>210</v>
-      </c>
-      <c r="E98">
+        <v>209</v>
+      </c>
+      <c r="E98" s="1">
         <v>10</v>
       </c>
       <c r="F98">
@@ -3150,12 +3179,12 @@
         <v>24151182</v>
       </c>
       <c r="B99" t="s">
-        <v>211</v>
-      </c>
-      <c r="D99">
+        <v>210</v>
+      </c>
+      <c r="D99" s="1">
         <v>1</v>
       </c>
-      <c r="E99">
+      <c r="E99" s="1">
         <v>4.5</v>
       </c>
       <c r="F99">
@@ -3164,18 +3193,18 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
+        <v>211</v>
+      </c>
+      <c r="B100" t="s">
         <v>212</v>
       </c>
-      <c r="B100" t="s">
+      <c r="C100" t="s">
         <v>213</v>
       </c>
-      <c r="C100" t="s">
-        <v>214</v>
-      </c>
-      <c r="D100">
+      <c r="D100" s="1">
         <v>0.85</v>
       </c>
-      <c r="E100">
+      <c r="E100" s="1">
         <v>2</v>
       </c>
       <c r="F100">
@@ -3184,12 +3213,12 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
+        <v>214</v>
+      </c>
+      <c r="B101" t="s">
         <v>215</v>
       </c>
-      <c r="B101" t="s">
-        <v>216</v>
-      </c>
-      <c r="E101">
+      <c r="E101" s="1">
         <v>8</v>
       </c>
       <c r="F101">
@@ -3201,9 +3230,9 @@
         <v>39103519</v>
       </c>
       <c r="B102" t="s">
-        <v>217</v>
-      </c>
-      <c r="E102">
+        <v>216</v>
+      </c>
+      <c r="E102" s="1">
         <v>3</v>
       </c>
       <c r="F102">
@@ -3212,18 +3241,18 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
+        <v>217</v>
+      </c>
+      <c r="B103" t="s">
         <v>218</v>
       </c>
-      <c r="B103" t="s">
+      <c r="C103" t="s">
         <v>219</v>
       </c>
-      <c r="C103" t="s">
-        <v>220</v>
-      </c>
-      <c r="D103">
+      <c r="D103" s="1">
         <v>7.9999479999999998</v>
       </c>
-      <c r="E103">
+      <c r="E103" s="1">
         <v>12</v>
       </c>
       <c r="F103">
@@ -3235,15 +3264,15 @@
         <v>3534</v>
       </c>
       <c r="B104" t="s">
+        <v>220</v>
+      </c>
+      <c r="C104" t="s">
         <v>221</v>
       </c>
-      <c r="C104" t="s">
-        <v>222</v>
-      </c>
-      <c r="D104">
+      <c r="D104" s="1">
         <v>2.3165</v>
       </c>
-      <c r="E104">
+      <c r="E104" s="1">
         <v>5</v>
       </c>
       <c r="F104">
@@ -3252,12 +3281,12 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
+        <v>222</v>
+      </c>
+      <c r="C105" t="s">
         <v>223</v>
       </c>
-      <c r="C105" t="s">
-        <v>224</v>
-      </c>
-      <c r="E105">
+      <c r="E105" s="1">
         <v>6.5</v>
       </c>
       <c r="F105">
@@ -3266,9 +3295,9 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
-        <v>225</v>
-      </c>
-      <c r="E106">
+        <v>224</v>
+      </c>
+      <c r="E106" s="1">
         <v>8.5</v>
       </c>
       <c r="F106">
@@ -3280,12 +3309,12 @@
         <v>243341</v>
       </c>
       <c r="B107" t="s">
-        <v>226</v>
-      </c>
-      <c r="D107">
+        <v>225</v>
+      </c>
+      <c r="D107" s="1">
         <v>3.8420000000000001</v>
       </c>
-      <c r="E107">
+      <c r="E107" s="1">
         <v>6.5</v>
       </c>
       <c r="F107">
@@ -3294,9 +3323,9 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
-        <v>227</v>
-      </c>
-      <c r="E108">
+        <v>226</v>
+      </c>
+      <c r="E108" s="1">
         <v>7.5</v>
       </c>
       <c r="F108">
@@ -3305,9 +3334,9 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
-        <v>228</v>
-      </c>
-      <c r="E109">
+        <v>227</v>
+      </c>
+      <c r="E109" s="1">
         <v>33</v>
       </c>
       <c r="F109">
@@ -3316,18 +3345,18 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
+        <v>228</v>
+      </c>
+      <c r="B110" t="s">
         <v>229</v>
       </c>
-      <c r="B110" t="s">
+      <c r="C110" t="s">
         <v>230</v>
       </c>
-      <c r="C110" t="s">
-        <v>231</v>
-      </c>
-      <c r="D110">
+      <c r="D110" s="1">
         <v>1.2543</v>
       </c>
-      <c r="E110">
+      <c r="E110" s="1">
         <v>3</v>
       </c>
       <c r="F110">
@@ -3336,12 +3365,12 @@
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
+        <v>231</v>
+      </c>
+      <c r="B111" t="s">
         <v>232</v>
       </c>
-      <c r="B111" t="s">
-        <v>233</v>
-      </c>
-      <c r="E111">
+      <c r="E111" s="1">
         <v>3</v>
       </c>
       <c r="F111">
@@ -3350,15 +3379,15 @@
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
+        <v>233</v>
+      </c>
+      <c r="B112" t="s">
         <v>234</v>
       </c>
-      <c r="B112" t="s">
-        <v>235</v>
-      </c>
-      <c r="D112">
+      <c r="D112" s="1">
         <v>4</v>
       </c>
-      <c r="E112">
+      <c r="E112" s="1">
         <v>12</v>
       </c>
       <c r="F112">
@@ -3367,9 +3396,9 @@
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
-        <v>236</v>
-      </c>
-      <c r="E113">
+        <v>235</v>
+      </c>
+      <c r="E113" s="1">
         <v>85</v>
       </c>
       <c r="F113">
@@ -3378,18 +3407,18 @@
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
+        <v>236</v>
+      </c>
+      <c r="B114" t="s">
         <v>237</v>
       </c>
-      <c r="B114" t="s">
+      <c r="C114" t="s">
         <v>238</v>
       </c>
-      <c r="C114" t="s">
-        <v>239</v>
-      </c>
-      <c r="D114">
+      <c r="D114" s="1">
         <v>12.999972</v>
       </c>
-      <c r="E114">
+      <c r="E114" s="1">
         <v>23</v>
       </c>
       <c r="F114">
@@ -3401,12 +3430,12 @@
         <v>6358129153</v>
       </c>
       <c r="B115" t="s">
-        <v>240</v>
-      </c>
-      <c r="D115">
+        <v>239</v>
+      </c>
+      <c r="D115" s="1">
         <v>8.7010000000000004E-2</v>
       </c>
-      <c r="E115">
+      <c r="E115" s="1">
         <v>0.25</v>
       </c>
       <c r="F115">
@@ -3418,12 +3447,12 @@
         <v>6358129193</v>
       </c>
       <c r="B116" t="s">
-        <v>241</v>
-      </c>
-      <c r="D116">
+        <v>240</v>
+      </c>
+      <c r="D116" s="1">
         <v>8.7010000000000004E-2</v>
       </c>
-      <c r="E116">
+      <c r="E116" s="1">
         <v>0.25</v>
       </c>
       <c r="F116">
@@ -3432,12 +3461,12 @@
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
+        <v>241</v>
+      </c>
+      <c r="B117" t="s">
         <v>242</v>
       </c>
-      <c r="B117" t="s">
-        <v>243</v>
-      </c>
-      <c r="E117">
+      <c r="E117" s="1">
         <v>65</v>
       </c>
       <c r="F117">
@@ -3446,9 +3475,9 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
-        <v>244</v>
-      </c>
-      <c r="E118">
+        <v>243</v>
+      </c>
+      <c r="E118" s="1">
         <v>70</v>
       </c>
       <c r="F118">
@@ -3457,15 +3486,15 @@
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
+        <v>244</v>
+      </c>
+      <c r="B119" t="s">
         <v>245</v>
       </c>
-      <c r="B119" t="s">
+      <c r="C119" t="s">
         <v>246</v>
       </c>
-      <c r="C119" t="s">
-        <v>247</v>
-      </c>
-      <c r="E119">
+      <c r="E119" s="1">
         <v>24</v>
       </c>
       <c r="F119">
@@ -3474,15 +3503,15 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
+        <v>247</v>
+      </c>
+      <c r="B120" t="s">
         <v>248</v>
       </c>
-      <c r="B120" t="s">
-        <v>249</v>
-      </c>
-      <c r="D120">
+      <c r="D120" s="1">
         <v>23</v>
       </c>
-      <c r="E120">
+      <c r="E120" s="1">
         <v>37</v>
       </c>
       <c r="F120">
@@ -3491,15 +3520,15 @@
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
+        <v>249</v>
+      </c>
+      <c r="B121" t="s">
         <v>250</v>
       </c>
-      <c r="B121" t="s">
-        <v>251</v>
-      </c>
-      <c r="D121">
+      <c r="D121" s="1">
         <v>26.5</v>
       </c>
-      <c r="E121">
+      <c r="E121" s="1">
         <v>37</v>
       </c>
       <c r="F121">
@@ -3508,9 +3537,9 @@
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
-        <v>252</v>
-      </c>
-      <c r="E122">
+        <v>251</v>
+      </c>
+      <c r="E122" s="1">
         <v>90</v>
       </c>
       <c r="F122">
@@ -3519,12 +3548,12 @@
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
+        <v>252</v>
+      </c>
+      <c r="C123" t="s">
         <v>253</v>
       </c>
-      <c r="C123" t="s">
-        <v>254</v>
-      </c>
-      <c r="E123">
+      <c r="E123" s="1">
         <v>12</v>
       </c>
       <c r="F123">
@@ -3533,15 +3562,15 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
+        <v>254</v>
+      </c>
+      <c r="B124" t="s">
         <v>255</v>
       </c>
-      <c r="B124" t="s">
+      <c r="C124" t="s">
         <v>256</v>
       </c>
-      <c r="C124" t="s">
-        <v>257</v>
-      </c>
-      <c r="E124">
+      <c r="E124" s="1">
         <v>12</v>
       </c>
       <c r="F124">
@@ -3550,15 +3579,15 @@
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
+        <v>257</v>
+      </c>
+      <c r="B125" t="s">
         <v>258</v>
       </c>
-      <c r="B125" t="s">
-        <v>259</v>
-      </c>
-      <c r="D125">
+      <c r="D125" s="1">
         <v>5.8872999999999998</v>
       </c>
-      <c r="E125">
+      <c r="E125" s="1">
         <v>12</v>
       </c>
       <c r="F125">
@@ -3567,15 +3596,15 @@
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
+        <v>259</v>
+      </c>
+      <c r="B126" t="s">
         <v>260</v>
       </c>
-      <c r="B126" t="s">
-        <v>261</v>
-      </c>
-      <c r="D126">
+      <c r="D126" s="1">
         <v>5.7968999999999991</v>
       </c>
-      <c r="E126">
+      <c r="E126" s="1">
         <v>12</v>
       </c>
       <c r="F126">
@@ -3584,9 +3613,9 @@
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
-        <v>262</v>
-      </c>
-      <c r="E127">
+        <v>261</v>
+      </c>
+      <c r="E127" s="1">
         <v>4</v>
       </c>
       <c r="F127">
@@ -3595,12 +3624,12 @@
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
+        <v>262</v>
+      </c>
+      <c r="C128" t="s">
         <v>263</v>
       </c>
-      <c r="C128" t="s">
-        <v>264</v>
-      </c>
-      <c r="E128">
+      <c r="E128" s="1">
         <v>20</v>
       </c>
       <c r="F128">
@@ -3609,12 +3638,12 @@
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
+        <v>264</v>
+      </c>
+      <c r="C129" t="s">
         <v>265</v>
       </c>
-      <c r="C129" t="s">
-        <v>266</v>
-      </c>
-      <c r="E129">
+      <c r="E129" s="1">
         <v>14.5</v>
       </c>
       <c r="F129">
@@ -3623,18 +3652,18 @@
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
+        <v>266</v>
+      </c>
+      <c r="B130" t="s">
         <v>267</v>
       </c>
-      <c r="B130" t="s">
+      <c r="C130" t="s">
         <v>268</v>
       </c>
-      <c r="C130" t="s">
-        <v>269</v>
-      </c>
-      <c r="D130">
+      <c r="D130" s="1">
         <v>14.995100000000001</v>
       </c>
-      <c r="E130">
+      <c r="E130" s="1">
         <v>23</v>
       </c>
       <c r="F130">
@@ -3643,12 +3672,12 @@
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B131" t="s">
+        <v>269</v>
+      </c>
+      <c r="C131" t="s">
         <v>270</v>
       </c>
-      <c r="C131" t="s">
-        <v>271</v>
-      </c>
-      <c r="E131">
+      <c r="E131" s="1">
         <v>15</v>
       </c>
       <c r="F131">
@@ -3657,18 +3686,18 @@
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
+        <v>271</v>
+      </c>
+      <c r="B132" t="s">
         <v>272</v>
       </c>
-      <c r="B132" t="s">
+      <c r="C132" t="s">
         <v>273</v>
       </c>
-      <c r="C132" t="s">
-        <v>274</v>
-      </c>
-      <c r="D132">
+      <c r="D132" s="1">
         <v>11</v>
       </c>
-      <c r="E132">
+      <c r="E132" s="1">
         <v>14.5</v>
       </c>
       <c r="F132">
@@ -3680,12 +3709,12 @@
         <v>4082300618280</v>
       </c>
       <c r="B133" t="s">
+        <v>274</v>
+      </c>
+      <c r="C133" t="s">
         <v>275</v>
       </c>
-      <c r="C133" t="s">
-        <v>276</v>
-      </c>
-      <c r="E133">
+      <c r="E133" s="1">
         <v>8</v>
       </c>
       <c r="F133">
@@ -3694,15 +3723,15 @@
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
+        <v>276</v>
+      </c>
+      <c r="B134" t="s">
         <v>277</v>
       </c>
-      <c r="B134" t="s">
-        <v>278</v>
-      </c>
       <c r="C134" t="s">
-        <v>278</v>
-      </c>
-      <c r="E134">
+        <v>277</v>
+      </c>
+      <c r="E134" s="1">
         <v>6</v>
       </c>
       <c r="F134">
@@ -3711,15 +3740,15 @@
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
+        <v>278</v>
+      </c>
+      <c r="B135" t="s">
         <v>279</v>
       </c>
-      <c r="B135" t="s">
-        <v>280</v>
-      </c>
-      <c r="D135">
+      <c r="D135" s="1">
         <v>8</v>
       </c>
-      <c r="E135">
+      <c r="E135" s="1">
         <v>11</v>
       </c>
       <c r="F135">
@@ -3731,12 +3760,12 @@
         <v>224131009</v>
       </c>
       <c r="B136" t="s">
+        <v>280</v>
+      </c>
+      <c r="C136" t="s">
         <v>281</v>
       </c>
-      <c r="C136" t="s">
-        <v>282</v>
-      </c>
-      <c r="E136">
+      <c r="E136" s="1">
         <v>8.5</v>
       </c>
       <c r="F136">
@@ -3745,9 +3774,9 @@
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B137" t="s">
-        <v>283</v>
-      </c>
-      <c r="E137">
+        <v>282</v>
+      </c>
+      <c r="E137" s="1">
         <v>45</v>
       </c>
       <c r="F137">
@@ -3756,15 +3785,15 @@
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
+        <v>283</v>
+      </c>
+      <c r="B138" t="s">
         <v>284</v>
       </c>
-      <c r="B138" t="s">
-        <v>285</v>
-      </c>
-      <c r="D138">
+      <c r="D138" s="1">
         <v>16.79</v>
       </c>
-      <c r="E138">
+      <c r="E138" s="1">
         <v>28</v>
       </c>
       <c r="F138">
@@ -3776,9 +3805,9 @@
         <v>2841200201</v>
       </c>
       <c r="B139" t="s">
-        <v>286</v>
-      </c>
-      <c r="E139">
+        <v>285</v>
+      </c>
+      <c r="E139" s="1">
         <v>35</v>
       </c>
       <c r="F139">
@@ -3790,9 +3819,9 @@
         <v>2841200301</v>
       </c>
       <c r="B140" t="s">
-        <v>287</v>
-      </c>
-      <c r="E140">
+        <v>286</v>
+      </c>
+      <c r="E140" s="1">
         <v>35</v>
       </c>
       <c r="F140">
@@ -3801,15 +3830,15 @@
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
+        <v>287</v>
+      </c>
+      <c r="B141" t="s">
         <v>288</v>
       </c>
-      <c r="B141" t="s">
-        <v>289</v>
-      </c>
-      <c r="D141">
+      <c r="D141" s="1">
         <v>12</v>
       </c>
-      <c r="E141">
+      <c r="E141" s="1">
         <v>18</v>
       </c>
       <c r="F141">
@@ -3818,15 +3847,15 @@
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
+        <v>289</v>
+      </c>
+      <c r="B142" t="s">
         <v>290</v>
       </c>
-      <c r="B142" t="s">
-        <v>291</v>
-      </c>
-      <c r="D142">
+      <c r="D142" s="1">
         <v>12</v>
       </c>
-      <c r="E142">
+      <c r="E142" s="1">
         <v>18</v>
       </c>
       <c r="F142">
@@ -3835,18 +3864,18 @@
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
+        <v>291</v>
+      </c>
+      <c r="B143" t="s">
         <v>292</v>
       </c>
-      <c r="B143" t="s">
+      <c r="C143" t="s">
         <v>293</v>
       </c>
-      <c r="C143" t="s">
-        <v>294</v>
-      </c>
-      <c r="D143">
+      <c r="D143" s="1">
         <v>1</v>
       </c>
-      <c r="E143">
+      <c r="E143" s="1">
         <v>3</v>
       </c>
       <c r="F143">
@@ -3855,9 +3884,9 @@
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
-        <v>295</v>
-      </c>
-      <c r="E144">
+        <v>294</v>
+      </c>
+      <c r="E144" s="1">
         <v>3.5</v>
       </c>
       <c r="F144">
@@ -3866,12 +3895,12 @@
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
+        <v>295</v>
+      </c>
+      <c r="B145" t="s">
         <v>296</v>
       </c>
-      <c r="B145" t="s">
-        <v>297</v>
-      </c>
-      <c r="E145">
+      <c r="E145" s="1">
         <v>97</v>
       </c>
       <c r="F145">
@@ -3880,18 +3909,18 @@
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
+        <v>297</v>
+      </c>
+      <c r="B146" t="s">
         <v>298</v>
       </c>
-      <c r="B146" t="s">
+      <c r="C146" t="s">
         <v>299</v>
       </c>
-      <c r="C146" t="s">
-        <v>300</v>
-      </c>
-      <c r="D146">
+      <c r="D146" s="1">
         <v>18.5</v>
       </c>
-      <c r="E146">
+      <c r="E146" s="1">
         <v>23</v>
       </c>
       <c r="F146">
@@ -3900,12 +3929,12 @@
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
+        <v>300</v>
+      </c>
+      <c r="B147" t="s">
         <v>301</v>
       </c>
-      <c r="B147" t="s">
-        <v>302</v>
-      </c>
-      <c r="E147">
+      <c r="E147" s="1">
         <v>30</v>
       </c>
       <c r="F147">
@@ -3914,15 +3943,15 @@
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
+        <v>302</v>
+      </c>
+      <c r="B148" t="s">
         <v>303</v>
       </c>
-      <c r="B148" t="s">
+      <c r="C148" t="s">
         <v>304</v>
       </c>
-      <c r="C148" t="s">
-        <v>305</v>
-      </c>
-      <c r="E148">
+      <c r="E148" s="1">
         <v>10</v>
       </c>
       <c r="F148">
@@ -3931,15 +3960,15 @@
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
+        <v>305</v>
+      </c>
+      <c r="B149" t="s">
         <v>306</v>
       </c>
-      <c r="B149" t="s">
-        <v>307</v>
-      </c>
-      <c r="D149">
+      <c r="D149" s="1">
         <v>0.75</v>
       </c>
-      <c r="E149">
+      <c r="E149" s="1">
         <v>3</v>
       </c>
       <c r="F149">
@@ -3948,18 +3977,18 @@
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
+        <v>307</v>
+      </c>
+      <c r="B150" t="s">
         <v>308</v>
       </c>
-      <c r="B150" t="s">
+      <c r="C150" t="s">
         <v>309</v>
       </c>
-      <c r="C150" t="s">
-        <v>310</v>
-      </c>
-      <c r="D150">
+      <c r="D150" s="1">
         <v>1</v>
       </c>
-      <c r="E150">
+      <c r="E150" s="1">
         <v>2</v>
       </c>
       <c r="F150">
@@ -3971,9 +4000,9 @@
         <v>5164</v>
       </c>
       <c r="B151" t="s">
-        <v>311</v>
-      </c>
-      <c r="E151">
+        <v>310</v>
+      </c>
+      <c r="E151" s="1">
         <v>32.5</v>
       </c>
       <c r="F151">
@@ -3982,15 +4011,15 @@
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
+        <v>311</v>
+      </c>
+      <c r="B152" t="s">
         <v>312</v>
       </c>
-      <c r="B152" t="s">
-        <v>313</v>
-      </c>
-      <c r="D152">
+      <c r="D152" s="1">
         <v>23.5</v>
       </c>
-      <c r="E152">
+      <c r="E152" s="1">
         <v>32.5</v>
       </c>
       <c r="F152">
@@ -4002,9 +4031,9 @@
         <v>22131018</v>
       </c>
       <c r="B153" t="s">
-        <v>314</v>
-      </c>
-      <c r="E153">
+        <v>313</v>
+      </c>
+      <c r="E153" s="1">
         <v>4</v>
       </c>
       <c r="F153">
@@ -4013,9 +4042,9 @@
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
-        <v>315</v>
-      </c>
-      <c r="E154">
+        <v>314</v>
+      </c>
+      <c r="E154" s="1">
         <v>8.5</v>
       </c>
       <c r="F154">
@@ -4024,9 +4053,9 @@
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
-        <v>316</v>
-      </c>
-      <c r="E155">
+        <v>315</v>
+      </c>
+      <c r="E155" s="1">
         <v>7</v>
       </c>
       <c r="F155">
@@ -4035,18 +4064,18 @@
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
+        <v>316</v>
+      </c>
+      <c r="B156" t="s">
         <v>317</v>
       </c>
-      <c r="B156" t="s">
+      <c r="C156" t="s">
         <v>318</v>
       </c>
-      <c r="C156" t="s">
-        <v>319</v>
-      </c>
-      <c r="D156">
+      <c r="D156" s="1">
         <v>1.25</v>
       </c>
-      <c r="E156">
+      <c r="E156" s="1">
         <v>4</v>
       </c>
       <c r="F156">
@@ -4055,9 +4084,9 @@
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
-        <v>320</v>
-      </c>
-      <c r="E157">
+        <v>319</v>
+      </c>
+      <c r="E157" s="1">
         <v>4</v>
       </c>
       <c r="F157">
@@ -4066,15 +4095,15 @@
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
+        <v>320</v>
+      </c>
+      <c r="B158" t="s">
         <v>321</v>
       </c>
-      <c r="B158" t="s">
-        <v>322</v>
-      </c>
-      <c r="D158">
+      <c r="D158" s="1">
         <v>13.71688</v>
       </c>
-      <c r="E158">
+      <c r="E158" s="1">
         <v>24</v>
       </c>
       <c r="F158">
@@ -4083,15 +4112,15 @@
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
+        <v>322</v>
+      </c>
+      <c r="B159" t="s">
         <v>323</v>
       </c>
-      <c r="B159" t="s">
-        <v>324</v>
-      </c>
-      <c r="D159">
+      <c r="D159" s="1">
         <v>0.64410000000000001</v>
       </c>
-      <c r="E159">
+      <c r="E159" s="1">
         <v>1</v>
       </c>
       <c r="F159">
@@ -4103,12 +4132,12 @@
         <v>3424</v>
       </c>
       <c r="B160" t="s">
+        <v>324</v>
+      </c>
+      <c r="C160" t="s">
         <v>325</v>
       </c>
-      <c r="C160" t="s">
-        <v>326</v>
-      </c>
-      <c r="E160">
+      <c r="E160" s="1">
         <v>6</v>
       </c>
       <c r="F160">
@@ -4117,18 +4146,18 @@
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
+        <v>326</v>
+      </c>
+      <c r="B161" t="s">
         <v>327</v>
       </c>
-      <c r="B161" t="s">
+      <c r="C161" t="s">
         <v>328</v>
       </c>
-      <c r="C161" t="s">
-        <v>329</v>
-      </c>
-      <c r="D161">
+      <c r="D161" s="1">
         <v>7.5031999999999996</v>
       </c>
-      <c r="E161">
+      <c r="E161" s="1">
         <v>12</v>
       </c>
       <c r="F161">
@@ -4137,15 +4166,15 @@
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
+        <v>329</v>
+      </c>
+      <c r="B162" t="s">
         <v>330</v>
       </c>
-      <c r="B162" t="s">
-        <v>331</v>
-      </c>
-      <c r="D162">
+      <c r="D162" s="1">
         <v>8.4862999999999982</v>
       </c>
-      <c r="E162">
+      <c r="E162" s="1">
         <v>13.5</v>
       </c>
       <c r="F162">
@@ -4154,9 +4183,9 @@
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B163" t="s">
-        <v>332</v>
-      </c>
-      <c r="E163">
+        <v>331</v>
+      </c>
+      <c r="E163" s="1">
         <v>12</v>
       </c>
       <c r="F163">
@@ -4165,15 +4194,15 @@
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
+        <v>332</v>
+      </c>
+      <c r="B164" t="s">
         <v>333</v>
       </c>
-      <c r="B164" t="s">
-        <v>334</v>
-      </c>
-      <c r="D164">
+      <c r="D164" s="1">
         <v>8.904399999999999</v>
       </c>
-      <c r="E164">
+      <c r="E164" s="1">
         <v>13.5</v>
       </c>
       <c r="F164">
@@ -4182,15 +4211,15 @@
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
+        <v>334</v>
+      </c>
+      <c r="B165" t="s">
         <v>335</v>
       </c>
-      <c r="B165" t="s">
+      <c r="C165" t="s">
         <v>336</v>
       </c>
-      <c r="C165" t="s">
-        <v>337</v>
-      </c>
-      <c r="E165">
+      <c r="E165" s="1">
         <v>10</v>
       </c>
       <c r="F165">
@@ -4199,12 +4228,12 @@
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
+        <v>337</v>
+      </c>
+      <c r="B166" t="s">
         <v>338</v>
       </c>
-      <c r="B166" t="s">
-        <v>339</v>
-      </c>
-      <c r="D166">
+      <c r="D166" s="1">
         <v>3.5</v>
       </c>
       <c r="F166">
@@ -4213,15 +4242,15 @@
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
+        <v>339</v>
+      </c>
+      <c r="B167" t="s">
         <v>340</v>
       </c>
-      <c r="B167" t="s">
-        <v>341</v>
-      </c>
-      <c r="D167">
+      <c r="D167" s="1">
         <v>2</v>
       </c>
-      <c r="E167">
+      <c r="E167" s="1">
         <v>6</v>
       </c>
       <c r="F167">
@@ -4230,18 +4259,18 @@
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
+        <v>341</v>
+      </c>
+      <c r="B168" t="s">
         <v>342</v>
       </c>
-      <c r="B168" t="s">
+      <c r="C168" t="s">
         <v>343</v>
       </c>
-      <c r="C168" t="s">
-        <v>344</v>
-      </c>
-      <c r="D168">
+      <c r="D168" s="1">
         <v>0.85</v>
       </c>
-      <c r="E168">
+      <c r="E168" s="1">
         <v>3.5</v>
       </c>
       <c r="F168">
@@ -4253,15 +4282,15 @@
         <v>22151106</v>
       </c>
       <c r="B169" t="s">
+        <v>344</v>
+      </c>
+      <c r="C169" t="s">
         <v>345</v>
       </c>
-      <c r="C169" t="s">
-        <v>346</v>
-      </c>
-      <c r="D169">
+      <c r="D169" s="1">
         <v>21</v>
       </c>
-      <c r="E169">
+      <c r="E169" s="1">
         <v>24.5</v>
       </c>
       <c r="F169">
@@ -4270,12 +4299,12 @@
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
+        <v>346</v>
+      </c>
+      <c r="B170" t="s">
         <v>347</v>
       </c>
-      <c r="B170" t="s">
-        <v>348</v>
-      </c>
-      <c r="E170">
+      <c r="E170" s="1">
         <v>23</v>
       </c>
       <c r="F170">
@@ -4284,15 +4313,15 @@
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
+        <v>348</v>
+      </c>
+      <c r="B171" t="s">
         <v>349</v>
       </c>
-      <c r="B171" t="s">
-        <v>350</v>
-      </c>
-      <c r="D171">
+      <c r="D171" s="1">
         <v>5.5</v>
       </c>
-      <c r="E171">
+      <c r="E171" s="1">
         <v>9</v>
       </c>
       <c r="F171">
@@ -4301,15 +4330,15 @@
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
+        <v>350</v>
+      </c>
+      <c r="B172" t="s">
         <v>351</v>
       </c>
-      <c r="B172" t="s">
-        <v>352</v>
-      </c>
-      <c r="D172">
+      <c r="D172" s="1">
         <v>2</v>
       </c>
-      <c r="E172">
+      <c r="E172" s="1">
         <v>6</v>
       </c>
       <c r="F172">
@@ -4318,9 +4347,9 @@
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B173" t="s">
-        <v>353</v>
-      </c>
-      <c r="E173">
+        <v>352</v>
+      </c>
+      <c r="E173" s="1">
         <v>1</v>
       </c>
       <c r="F173">
@@ -4332,9 +4361,9 @@
         <v>4632</v>
       </c>
       <c r="B174" t="s">
-        <v>354</v>
-      </c>
-      <c r="E174">
+        <v>353</v>
+      </c>
+      <c r="E174" s="1">
         <v>4</v>
       </c>
       <c r="F174">
@@ -4343,9 +4372,9 @@
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B175" t="s">
-        <v>355</v>
-      </c>
-      <c r="E175">
+        <v>354</v>
+      </c>
+      <c r="E175" s="1">
         <v>4</v>
       </c>
       <c r="F175">
@@ -4354,15 +4383,15 @@
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
+        <v>355</v>
+      </c>
+      <c r="B176" t="s">
         <v>356</v>
       </c>
-      <c r="B176" t="s">
-        <v>357</v>
-      </c>
-      <c r="D176">
+      <c r="D176" s="1">
         <v>2</v>
       </c>
-      <c r="E176">
+      <c r="E176" s="1">
         <v>5</v>
       </c>
       <c r="F176">
@@ -4374,12 +4403,12 @@
         <v>24151175</v>
       </c>
       <c r="B177" t="s">
-        <v>358</v>
-      </c>
-      <c r="D177">
+        <v>357</v>
+      </c>
+      <c r="D177" s="1">
         <v>2.75</v>
       </c>
-      <c r="E177">
+      <c r="E177" s="1">
         <v>6.5</v>
       </c>
       <c r="F177">
@@ -4391,12 +4420,12 @@
         <v>24151179</v>
       </c>
       <c r="B178" t="s">
-        <v>359</v>
-      </c>
-      <c r="D178">
+        <v>358</v>
+      </c>
+      <c r="D178" s="1">
         <v>2.75</v>
       </c>
-      <c r="E178">
+      <c r="E178" s="1">
         <v>6.5</v>
       </c>
       <c r="F178">
@@ -4405,12 +4434,12 @@
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
+        <v>359</v>
+      </c>
+      <c r="B179" t="s">
         <v>360</v>
       </c>
-      <c r="B179" t="s">
-        <v>361</v>
-      </c>
-      <c r="E179">
+      <c r="E179" s="1">
         <v>6</v>
       </c>
       <c r="F179">
@@ -4422,9 +4451,9 @@
         <v>39193815</v>
       </c>
       <c r="B180" t="s">
-        <v>362</v>
-      </c>
-      <c r="E180">
+        <v>361</v>
+      </c>
+      <c r="E180" s="1">
         <v>2</v>
       </c>
       <c r="F180">
@@ -4433,12 +4462,12 @@
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B181" t="s">
+        <v>362</v>
+      </c>
+      <c r="C181" t="s">
         <v>363</v>
       </c>
-      <c r="C181" t="s">
-        <v>364</v>
-      </c>
-      <c r="E181">
+      <c r="E181" s="1">
         <v>50</v>
       </c>
       <c r="F181">

</xml_diff>

<commit_message>
Módulo de Entradas Refactorizado: Agrupación por factura, detalles expandibles, flujo proactivo de códigos para productos nuevos y optimización de navegación por teclado.
</commit_message>
<xml_diff>
--- a/Inventario Diciembre.xlsx
+++ b/Inventario Diciembre.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b751df8fdfd3fc6f/Documentos/GitHub/willianworkshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{3CCFD0E0-91E2-432E-9EC5-28D300F50351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{637AD33F-6749-437A-AA97-030EA40D7274}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{3CCFD0E0-91E2-432E-9EC5-28D300F50351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02D05870-8F6D-49E0-AF3E-93AC19F8AA9E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{36D6B9B6-F2BD-47F5-95D5-897B11381D8C}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="367">
   <si>
     <t>Codigo</t>
   </si>
@@ -1135,6 +1135,9 @@
   </si>
   <si>
     <t>Precio de costo</t>
+  </si>
+  <si>
+    <t>*</t>
   </si>
 </sst>
 </file>
@@ -1144,7 +1147,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1163,6 +1166,15 @@
       <b/>
       <i/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1190,7 +1202,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1200,6 +1212,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -1515,18 +1530,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{727700AC-25D3-4333-982B-13D5617599C9}">
-  <dimension ref="A1:F181"/>
+  <dimension ref="A1:G181"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="45.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1545,8 +1560,9 @@
       <c r="F1" s="2" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G1" s="5"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>3401502</v>
       </c>
@@ -1562,8 +1578,11 @@
       <c r="F2">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1579,8 +1598,11 @@
       <c r="F3">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G3" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1593,8 +1615,11 @@
       <c r="F4">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1607,8 +1632,11 @@
       <c r="F5">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>3406</v>
       </c>
@@ -1627,8 +1655,11 @@
       <c r="F6">
         <v>86</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G6" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>52240764</v>
       </c>
@@ -1644,8 +1675,11 @@
       <c r="F7">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>31101020</v>
       </c>
@@ -1661,8 +1695,11 @@
       <c r="F8">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G8" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>16</v>
       </c>
@@ -1672,8 +1709,11 @@
       <c r="F9">
         <v>27</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G9" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>17</v>
       </c>
@@ -1683,8 +1723,11 @@
       <c r="F10">
         <v>26</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G10" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>18</v>
       </c>
@@ -1694,8 +1737,11 @@
       <c r="F11">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G11" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>19</v>
       </c>
@@ -1705,8 +1751,11 @@
       <c r="F12">
         <v>4</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G12" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>39143520</v>
       </c>
@@ -1725,8 +1774,11 @@
       <c r="F13">
         <v>30</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G13" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>22</v>
       </c>
@@ -1736,8 +1788,11 @@
       <c r="F14">
         <v>20</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G14" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>23</v>
       </c>
@@ -1747,8 +1802,11 @@
       <c r="F15">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G15" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>24</v>
       </c>
@@ -1758,8 +1816,11 @@
       <c r="F16">
         <v>5</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G16" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>25</v>
       </c>
@@ -1778,8 +1839,11 @@
       <c r="F17">
         <v>9</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G17" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -1798,8 +1862,11 @@
       <c r="F18">
         <v>5</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G18" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -1818,8 +1885,11 @@
       <c r="F19">
         <v>9</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G19" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>34</v>
       </c>
@@ -1832,8 +1902,11 @@
       <c r="F20">
         <v>6</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G20" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>36</v>
       </c>
@@ -1846,8 +1919,11 @@
       <c r="F21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G21" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>482680181601</v>
       </c>
@@ -1866,8 +1942,11 @@
       <c r="F22">
         <v>502</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G22" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>40</v>
       </c>
@@ -1883,8 +1962,11 @@
       <c r="F23">
         <v>6</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G23" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>42</v>
       </c>
@@ -1904,7 +1986,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>45</v>
       </c>
@@ -1920,8 +2002,11 @@
       <c r="F25">
         <v>15</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G25" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>47</v>
       </c>
@@ -1937,8 +2022,11 @@
       <c r="F26">
         <v>60</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G26" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>50</v>
       </c>
@@ -1954,8 +2042,11 @@
       <c r="F27">
         <v>6</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G27" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>52</v>
       </c>
@@ -1974,8 +2065,11 @@
       <c r="F28">
         <v>29</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G28" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>55</v>
       </c>
@@ -1994,8 +2088,11 @@
       <c r="F29">
         <v>11</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G29" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>58</v>
       </c>
@@ -2011,8 +2108,11 @@
       <c r="F30">
         <v>12</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G30" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>61</v>
       </c>
@@ -2028,8 +2128,11 @@
       <c r="F31">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G31" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>63</v>
       </c>
@@ -2045,8 +2148,11 @@
       <c r="F32">
         <v>5</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G32" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>65</v>
       </c>
@@ -2062,8 +2168,11 @@
       <c r="F33">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G33" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>67</v>
       </c>
@@ -2079,8 +2188,11 @@
       <c r="F34">
         <v>2</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G34" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>69</v>
       </c>
@@ -2096,8 +2208,11 @@
       <c r="F35">
         <v>5</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G35" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>71</v>
       </c>
@@ -2116,8 +2231,11 @@
       <c r="F36">
         <v>31</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G36" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>74</v>
       </c>
@@ -2133,8 +2251,11 @@
       <c r="F37">
         <v>28</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G37" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>76</v>
       </c>
@@ -2150,8 +2271,11 @@
       <c r="F38">
         <v>19</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G38" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>78</v>
       </c>
@@ -2170,8 +2294,11 @@
       <c r="F39">
         <v>64</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G39" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>81</v>
       </c>
@@ -2184,8 +2311,11 @@
       <c r="F40">
         <v>13</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G40" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>83</v>
       </c>
@@ -2198,8 +2328,11 @@
       <c r="F41">
         <v>13</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G41" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>85</v>
       </c>
@@ -2209,8 +2342,11 @@
       <c r="F42">
         <v>9</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G42" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>86</v>
       </c>
@@ -2220,8 +2356,11 @@
       <c r="F43">
         <v>27</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G43" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>87</v>
       </c>
@@ -2234,8 +2373,11 @@
       <c r="F44">
         <v>8</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G44" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>89</v>
       </c>
@@ -2255,7 +2397,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>92</v>
       </c>
@@ -2271,8 +2413,11 @@
       <c r="F46">
         <v>13</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G46" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>94</v>
       </c>
@@ -2292,7 +2437,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>97</v>
       </c>
@@ -2312,7 +2457,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>100</v>
       </c>
@@ -2329,7 +2474,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>102</v>
       </c>
@@ -2345,8 +2490,11 @@
       <c r="F50">
         <v>5</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G50" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>104</v>
       </c>
@@ -2359,8 +2507,11 @@
       <c r="F51">
         <v>3</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G51" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>106</v>
       </c>
@@ -2379,8 +2530,11 @@
       <c r="F52">
         <v>10</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G52" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>4841</v>
       </c>
@@ -2399,8 +2553,11 @@
       <c r="F53">
         <v>2</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G53" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>111</v>
       </c>
@@ -2417,7 +2574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
         <v>113</v>
       </c>
@@ -2427,8 +2584,11 @@
       <c r="F55">
         <v>3</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G55" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>114</v>
       </c>
@@ -2441,8 +2601,11 @@
       <c r="F56">
         <v>4</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G56" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>116</v>
       </c>
@@ -2455,8 +2618,11 @@
       <c r="F57">
         <v>9</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G57" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>1650101601</v>
       </c>
@@ -2472,8 +2638,11 @@
       <c r="F58">
         <v>17</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G58" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>242477</v>
       </c>
@@ -2489,8 +2658,11 @@
       <c r="F59">
         <v>5</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G59" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>122</v>
       </c>
@@ -2509,8 +2681,11 @@
       <c r="F60">
         <v>3</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G60" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>125</v>
       </c>
@@ -2526,8 +2701,11 @@
       <c r="F61">
         <v>2</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G61" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>128</v>
       </c>
@@ -2546,8 +2724,11 @@
       <c r="F62">
         <v>3</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G62" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>131</v>
       </c>
@@ -2560,8 +2741,11 @@
       <c r="F63">
         <v>2</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G63" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>133</v>
       </c>
@@ -2577,8 +2761,11 @@
       <c r="F64">
         <v>12</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G64" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>135</v>
       </c>
@@ -2594,8 +2781,11 @@
       <c r="F65">
         <v>2</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G65" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>137</v>
       </c>
@@ -2611,8 +2801,11 @@
       <c r="F66">
         <v>5</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G66" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>139</v>
       </c>
@@ -2629,7 +2822,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>141</v>
       </c>
@@ -2648,8 +2841,11 @@
       <c r="F68">
         <v>1</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G68" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>144</v>
       </c>
@@ -2665,8 +2861,11 @@
       <c r="F69">
         <v>5</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G69" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
         <v>147</v>
       </c>
@@ -2679,8 +2878,11 @@
       <c r="F70">
         <v>14</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G70" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>148</v>
       </c>
@@ -2699,8 +2901,11 @@
       <c r="F71">
         <v>8</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G71" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>2871</v>
       </c>
@@ -2713,8 +2918,11 @@
       <c r="F72">
         <v>15</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G72" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>152</v>
       </c>
@@ -2733,8 +2941,11 @@
       <c r="F73">
         <v>7</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G73" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>155</v>
       </c>
@@ -2750,8 +2961,11 @@
       <c r="F74">
         <v>66</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G74" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>4092</v>
       </c>
@@ -2764,8 +2978,11 @@
       <c r="F75">
         <v>20</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G75" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>159</v>
       </c>
@@ -2784,8 +3001,11 @@
       <c r="F76">
         <v>5</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G76" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>28101110</v>
       </c>
@@ -2801,8 +3021,11 @@
       <c r="F77">
         <v>7</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G77" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
         <v>164</v>
       </c>
@@ -2815,8 +3038,11 @@
       <c r="F78">
         <v>49</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G78" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>166</v>
       </c>
@@ -2832,8 +3058,11 @@
       <c r="F79">
         <v>5</v>
       </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G79" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>168</v>
       </c>
@@ -2852,8 +3081,11 @@
       <c r="F80">
         <v>163</v>
       </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G80" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>171</v>
       </c>
@@ -2873,7 +3105,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>174</v>
       </c>
@@ -2892,8 +3124,11 @@
       <c r="F82">
         <v>133</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G82" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>177</v>
       </c>
@@ -2912,8 +3147,11 @@
       <c r="F83">
         <v>4</v>
       </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G83" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>180</v>
       </c>
@@ -2932,8 +3170,11 @@
       <c r="F84">
         <v>5</v>
       </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G84" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>6358129273</v>
       </c>
@@ -2950,7 +3191,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>6358129313</v>
       </c>
@@ -2967,7 +3208,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>185</v>
       </c>
@@ -2983,8 +3224,11 @@
       <c r="F87">
         <v>37</v>
       </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G87" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>52244040</v>
       </c>
@@ -3004,7 +3248,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>52210040</v>
       </c>
@@ -3017,8 +3261,11 @@
       <c r="F89">
         <v>11</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G89" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>190</v>
       </c>
@@ -3037,8 +3284,11 @@
       <c r="F90">
         <v>15</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G90" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>193</v>
       </c>
@@ -3057,8 +3307,11 @@
       <c r="F91">
         <v>8</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G91" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>196</v>
       </c>
@@ -3071,8 +3324,11 @@
       <c r="F92">
         <v>10</v>
       </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G92" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>198</v>
       </c>
@@ -3088,8 +3344,11 @@
       <c r="F93">
         <v>31</v>
       </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G93" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>200</v>
       </c>
@@ -3105,8 +3364,11 @@
       <c r="F94">
         <v>8</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G94" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>202</v>
       </c>
@@ -3125,8 +3387,11 @@
       <c r="F95">
         <v>15</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G95" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>205</v>
       </c>
@@ -3142,8 +3407,11 @@
       <c r="F96">
         <v>4</v>
       </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G96" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>207</v>
       </c>
@@ -3159,8 +3427,11 @@
       <c r="F97">
         <v>33</v>
       </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G97" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>4092</v>
       </c>
@@ -3173,8 +3444,11 @@
       <c r="F98">
         <v>10</v>
       </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G98" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>24151182</v>
       </c>
@@ -3190,8 +3464,11 @@
       <c r="F99">
         <v>5</v>
       </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G99" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>211</v>
       </c>
@@ -3211,7 +3488,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>214</v>
       </c>
@@ -3224,8 +3501,11 @@
       <c r="F101">
         <v>9</v>
       </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G101" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>39103519</v>
       </c>
@@ -3238,8 +3518,11 @@
       <c r="F102">
         <v>11</v>
       </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G102" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>217</v>
       </c>
@@ -3258,8 +3541,11 @@
       <c r="F103">
         <v>6</v>
       </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G103" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>3534</v>
       </c>
@@ -3278,8 +3564,11 @@
       <c r="F104">
         <v>63</v>
       </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G104" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
         <v>222</v>
       </c>
@@ -3292,8 +3581,11 @@
       <c r="F105">
         <v>7</v>
       </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G105" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
         <v>224</v>
       </c>
@@ -3303,8 +3595,11 @@
       <c r="F106">
         <v>17</v>
       </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G106" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>243341</v>
       </c>
@@ -3320,8 +3615,11 @@
       <c r="F107">
         <v>13</v>
       </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G107" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
         <v>226</v>
       </c>
@@ -3331,8 +3629,11 @@
       <c r="F108">
         <v>71</v>
       </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G108" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
         <v>227</v>
       </c>
@@ -3342,8 +3643,11 @@
       <c r="F109">
         <v>58</v>
       </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G109" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>228</v>
       </c>
@@ -3362,8 +3666,11 @@
       <c r="F110">
         <v>31</v>
       </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G110" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>231</v>
       </c>
@@ -3376,8 +3683,11 @@
       <c r="F111">
         <v>7</v>
       </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G111" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>233</v>
       </c>
@@ -3393,8 +3703,11 @@
       <c r="F112">
         <v>2</v>
       </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G112" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
         <v>235</v>
       </c>
@@ -3404,8 +3717,11 @@
       <c r="F113">
         <v>1</v>
       </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G113" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>236</v>
       </c>
@@ -3424,8 +3740,11 @@
       <c r="F114">
         <v>6</v>
       </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G114" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>6358129153</v>
       </c>
@@ -3442,7 +3761,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>6358129193</v>
       </c>
@@ -3459,7 +3778,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>241</v>
       </c>
@@ -3472,8 +3791,11 @@
       <c r="F117">
         <v>4</v>
       </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G117" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
         <v>243</v>
       </c>
@@ -3483,8 +3805,11 @@
       <c r="F118">
         <v>2</v>
       </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G118" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>244</v>
       </c>
@@ -3500,8 +3825,11 @@
       <c r="F119">
         <v>3</v>
       </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G119" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>247</v>
       </c>
@@ -3517,8 +3845,11 @@
       <c r="F120">
         <v>2</v>
       </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G120" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>249</v>
       </c>
@@ -3534,8 +3865,11 @@
       <c r="F121">
         <v>2</v>
       </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G121" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
         <v>251</v>
       </c>
@@ -3545,8 +3879,11 @@
       <c r="F122">
         <v>0</v>
       </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G122" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>252</v>
       </c>
@@ -3559,8 +3896,11 @@
       <c r="F123">
         <v>1</v>
       </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G123" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>254</v>
       </c>
@@ -3576,8 +3916,11 @@
       <c r="F124">
         <v>2</v>
       </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G124" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>257</v>
       </c>
@@ -3593,8 +3936,11 @@
       <c r="F125">
         <v>6</v>
       </c>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G125" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>259</v>
       </c>
@@ -3610,8 +3956,11 @@
       <c r="F126">
         <v>6</v>
       </c>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G126" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>261</v>
       </c>
@@ -3621,8 +3970,11 @@
       <c r="F127">
         <v>3</v>
       </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G127" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
         <v>262</v>
       </c>
@@ -3635,8 +3987,11 @@
       <c r="F128">
         <v>5</v>
       </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G128" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
         <v>264</v>
       </c>
@@ -3649,8 +4004,11 @@
       <c r="F129">
         <v>6</v>
       </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G129" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>266</v>
       </c>
@@ -3669,8 +4027,11 @@
       <c r="F130">
         <v>9</v>
       </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G130" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B131" t="s">
         <v>269</v>
       </c>
@@ -3683,8 +4044,11 @@
       <c r="F131">
         <v>2</v>
       </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G131" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>271</v>
       </c>
@@ -3703,8 +4067,11 @@
       <c r="F132">
         <v>3</v>
       </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G132" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>4082300618280</v>
       </c>
@@ -3720,8 +4087,11 @@
       <c r="F133">
         <v>9</v>
       </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G133" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>276</v>
       </c>
@@ -3737,8 +4107,11 @@
       <c r="F134">
         <v>60</v>
       </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G134" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>278</v>
       </c>
@@ -3754,8 +4127,11 @@
       <c r="F135">
         <v>5</v>
       </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G135" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>224131009</v>
       </c>
@@ -3771,8 +4147,11 @@
       <c r="F136">
         <v>8</v>
       </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G136" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B137" t="s">
         <v>282</v>
       </c>
@@ -3782,8 +4161,11 @@
       <c r="F137">
         <v>1</v>
       </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G137" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>283</v>
       </c>
@@ -3799,8 +4181,11 @@
       <c r="F138">
         <v>14</v>
       </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G138" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>2841200201</v>
       </c>
@@ -3813,8 +4198,11 @@
       <c r="F139">
         <v>2</v>
       </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G139" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>2841200301</v>
       </c>
@@ -3827,8 +4215,11 @@
       <c r="F140">
         <v>2</v>
       </c>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G140" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>287</v>
       </c>
@@ -3844,8 +4235,11 @@
       <c r="F141">
         <v>2</v>
       </c>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G141" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>289</v>
       </c>
@@ -3861,8 +4255,11 @@
       <c r="F142">
         <v>2</v>
       </c>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G142" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>291</v>
       </c>
@@ -3881,8 +4278,11 @@
       <c r="F143">
         <v>53</v>
       </c>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G143" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
         <v>294</v>
       </c>
@@ -3892,8 +4292,11 @@
       <c r="F144">
         <v>37</v>
       </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G144" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>295</v>
       </c>
@@ -3906,8 +4309,11 @@
       <c r="F145">
         <v>2</v>
       </c>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G145" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>297</v>
       </c>
@@ -3926,8 +4332,11 @@
       <c r="F146">
         <v>4</v>
       </c>
-    </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G146" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>300</v>
       </c>
@@ -3940,8 +4349,11 @@
       <c r="F147">
         <v>6</v>
       </c>
-    </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G147" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>302</v>
       </c>
@@ -3957,8 +4369,11 @@
       <c r="F148">
         <v>11</v>
       </c>
-    </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G148" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>305</v>
       </c>
@@ -3974,8 +4389,11 @@
       <c r="F149">
         <v>5</v>
       </c>
-    </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G149" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>307</v>
       </c>
@@ -3994,8 +4412,11 @@
       <c r="F150">
         <v>36</v>
       </c>
-    </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G150">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>5164</v>
       </c>
@@ -4008,8 +4429,11 @@
       <c r="F151">
         <v>0</v>
       </c>
-    </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G151" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>311</v>
       </c>
@@ -4025,8 +4449,11 @@
       <c r="F152">
         <v>4</v>
       </c>
-    </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G152" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>22131018</v>
       </c>
@@ -4039,8 +4466,11 @@
       <c r="F153">
         <v>10</v>
       </c>
-    </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G153" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
         <v>314</v>
       </c>
@@ -4050,8 +4480,11 @@
       <c r="F154">
         <v>2</v>
       </c>
-    </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G154" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
         <v>315</v>
       </c>
@@ -4061,8 +4494,11 @@
       <c r="F155">
         <v>9</v>
       </c>
-    </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G155" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>316</v>
       </c>
@@ -4081,8 +4517,11 @@
       <c r="F156">
         <v>14</v>
       </c>
-    </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G156" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
         <v>319</v>
       </c>
@@ -4092,8 +4531,11 @@
       <c r="F157">
         <v>21</v>
       </c>
-    </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G157" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>320</v>
       </c>
@@ -4109,8 +4551,11 @@
       <c r="F158">
         <v>2</v>
       </c>
-    </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G158" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>322</v>
       </c>
@@ -4126,8 +4571,11 @@
       <c r="F159">
         <v>82</v>
       </c>
-    </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G159" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>3424</v>
       </c>
@@ -4143,8 +4591,11 @@
       <c r="F160">
         <v>6</v>
       </c>
-    </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G160" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>326</v>
       </c>
@@ -4163,8 +4614,11 @@
       <c r="F161">
         <v>3</v>
       </c>
-    </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G161" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>329</v>
       </c>
@@ -4180,8 +4634,11 @@
       <c r="F162">
         <v>4</v>
       </c>
-    </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G162" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B163" t="s">
         <v>331</v>
       </c>
@@ -4192,7 +4649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>332</v>
       </c>
@@ -4208,8 +4665,11 @@
       <c r="F164">
         <v>4</v>
       </c>
-    </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G164" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>334</v>
       </c>
@@ -4225,8 +4685,11 @@
       <c r="F165">
         <v>5</v>
       </c>
-    </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G165" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>337</v>
       </c>
@@ -4240,7 +4703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>339</v>
       </c>
@@ -4256,8 +4719,11 @@
       <c r="F167">
         <v>8</v>
       </c>
-    </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G167" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>341</v>
       </c>
@@ -4276,8 +4742,11 @@
       <c r="F168">
         <v>5</v>
       </c>
-    </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G168" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>22151106</v>
       </c>
@@ -4296,8 +4765,11 @@
       <c r="F169">
         <v>2</v>
       </c>
-    </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G169" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>346</v>
       </c>
@@ -4310,8 +4782,11 @@
       <c r="F170">
         <v>1</v>
       </c>
-    </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G170" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>348</v>
       </c>
@@ -4327,8 +4802,11 @@
       <c r="F171">
         <v>14</v>
       </c>
-    </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G171" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>350</v>
       </c>
@@ -4344,8 +4822,11 @@
       <c r="F172">
         <v>5</v>
       </c>
-    </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G172" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B173" t="s">
         <v>352</v>
       </c>
@@ -4355,8 +4836,11 @@
       <c r="F173">
         <v>73</v>
       </c>
-    </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G173" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>4632</v>
       </c>
@@ -4369,8 +4853,11 @@
       <c r="F174">
         <v>5</v>
       </c>
-    </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G174" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B175" t="s">
         <v>354</v>
       </c>
@@ -4380,8 +4867,11 @@
       <c r="F175">
         <v>10</v>
       </c>
-    </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G175" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>355</v>
       </c>
@@ -4397,8 +4887,11 @@
       <c r="F176">
         <v>15</v>
       </c>
-    </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G176" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>24151175</v>
       </c>
@@ -4414,8 +4907,11 @@
       <c r="F177">
         <v>3</v>
       </c>
-    </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G177" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>24151179</v>
       </c>
@@ -4431,8 +4927,11 @@
       <c r="F178">
         <v>3</v>
       </c>
-    </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G178" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>359</v>
       </c>
@@ -4445,8 +4944,11 @@
       <c r="F179">
         <v>6</v>
       </c>
-    </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G179" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>39193815</v>
       </c>
@@ -4459,8 +4961,11 @@
       <c r="F180">
         <v>9</v>
       </c>
-    </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G180" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B181" t="s">
         <v>362</v>
       </c>
@@ -4472,6 +4977,9 @@
       </c>
       <c r="F181">
         <v>2</v>
+      </c>
+      <c r="G181" t="s">
+        <v>366</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización del sistema de inventario - mejoras en controladores y servicios
</commit_message>
<xml_diff>
--- a/Inventario Diciembre.xlsx
+++ b/Inventario Diciembre.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b751df8fdfd3fc6f/Documentos/GitHub/willianworkshop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Esteban\.gemini\antigravity\scratch\willianworkshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{3CCFD0E0-91E2-432E-9EC5-28D300F50351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C6DFEB3-F37C-480B-87BA-E1B3ABF70B7C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB1B7EEC-2C5E-47FE-89BD-FAC83BF93EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{36D6B9B6-F2BD-47F5-95D5-897B11381D8C}"/>
   </bookViews>
@@ -891,21 +891,6 @@
     <t>Volante solo Bajaj 175</t>
   </si>
   <si>
-    <t>CODIGO</t>
-  </si>
-  <si>
-    <t>DESCRIPCIONINVENTARIO</t>
-  </si>
-  <si>
-    <t>PRECIO COSTO</t>
-  </si>
-  <si>
-    <t>PRECIO VENTA</t>
-  </si>
-  <si>
-    <t>EXISTENCIA</t>
-  </si>
-  <si>
     <t>AB181012</t>
   </si>
   <si>
@@ -949,6 +934,21 @@
   </si>
   <si>
     <t>Tensor de cadena de tiempo</t>
+  </si>
+  <si>
+    <t>Codigo</t>
+  </si>
+  <si>
+    <t>Descripcion inventario</t>
+  </si>
+  <si>
+    <t>Precio costo</t>
+  </si>
+  <si>
+    <t>Precio de venta</t>
+  </si>
+  <si>
+    <t>Existencia</t>
   </si>
 </sst>
 </file>
@@ -1023,9 +1023,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1063,7 +1063,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1169,7 +1169,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1311,7 +1311,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1324,26 +1324,25 @@
   <cols>
     <col min="1" max="1" width="29.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="45.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>284</v>
+        <v>299</v>
       </c>
       <c r="B1" t="s">
-        <v>285</v>
+        <v>300</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>287</v>
+        <v>301</v>
+      </c>
+      <c r="D1" t="s">
+        <v>302</v>
       </c>
       <c r="E1" t="s">
-        <v>288</v>
+        <v>303</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -1356,7 +1355,7 @@
       <c r="C2" s="1">
         <v>7</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2">
         <v>12</v>
       </c>
       <c r="E2">
@@ -1373,7 +1372,7 @@
       <c r="C3" s="1">
         <v>10</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3">
         <v>15</v>
       </c>
       <c r="E3">
@@ -1387,7 +1386,7 @@
       <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4">
         <v>16</v>
       </c>
       <c r="E4">
@@ -1404,7 +1403,7 @@
       <c r="C5" s="1">
         <v>9.5000230000000006</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5">
         <v>16</v>
       </c>
       <c r="E5">
@@ -1421,7 +1420,7 @@
       <c r="C6" s="1">
         <v>0.19209999999999999</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6">
         <v>1</v>
       </c>
       <c r="E6">
@@ -1435,7 +1434,7 @@
       <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7">
         <v>20</v>
       </c>
       <c r="E7">
@@ -1452,7 +1451,7 @@
       <c r="C8" s="1">
         <v>3.5</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8">
         <v>7</v>
       </c>
       <c r="E8">
@@ -1461,12 +1460,12 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="B9" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9">
         <v>3</v>
       </c>
       <c r="E9">
@@ -1475,12 +1474,12 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10">
         <v>2</v>
       </c>
       <c r="E10">
@@ -1491,7 +1490,7 @@
       <c r="B11" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11">
         <v>6</v>
       </c>
       <c r="E11">
@@ -1502,7 +1501,7 @@
       <c r="B12" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12">
         <v>7</v>
       </c>
       <c r="E12">
@@ -1519,7 +1518,7 @@
       <c r="C13" s="1">
         <v>1.699972</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13">
         <v>5</v>
       </c>
       <c r="E13">
@@ -1528,7 +1527,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="B14" t="s">
         <v>15</v>
@@ -1536,7 +1535,7 @@
       <c r="C14" s="1">
         <v>4.1500000000000004</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14">
         <v>8</v>
       </c>
       <c r="E14">
@@ -1545,7 +1544,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
@@ -1553,7 +1552,7 @@
       <c r="C15" s="1">
         <v>10.34</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15">
         <v>13.5</v>
       </c>
       <c r="E15">
@@ -1564,7 +1563,7 @@
       <c r="B16" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16">
         <v>5</v>
       </c>
       <c r="E16">
@@ -1581,7 +1580,7 @@
       <c r="C17" s="1">
         <v>1.0508999999999999</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17">
         <v>3</v>
       </c>
       <c r="E17">
@@ -1598,7 +1597,7 @@
       <c r="C18" s="1">
         <v>1.0508999999999999</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18">
         <v>3</v>
       </c>
       <c r="E18">
@@ -1615,7 +1614,7 @@
       <c r="C19" s="1">
         <v>1.85</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19">
         <v>4</v>
       </c>
       <c r="E19">
@@ -1632,7 +1631,7 @@
       <c r="C20" s="1">
         <v>6.4999859999999998</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20">
         <v>13.5</v>
       </c>
       <c r="E20">
@@ -1643,7 +1642,7 @@
       <c r="B21" t="s">
         <v>26</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21">
         <v>3</v>
       </c>
       <c r="E21">
@@ -1660,7 +1659,7 @@
       <c r="C22" s="1">
         <v>0.23119799999999999</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22">
         <v>0.5</v>
       </c>
       <c r="E22">
@@ -1677,7 +1676,7 @@
       <c r="C23" s="1">
         <v>23</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23">
         <v>30</v>
       </c>
       <c r="E23">
@@ -1694,7 +1693,7 @@
       <c r="C24" s="1">
         <v>16.995200000000001</v>
       </c>
-      <c r="D24" s="1">
+      <c r="D24">
         <v>40</v>
       </c>
       <c r="E24">
@@ -1711,7 +1710,7 @@
       <c r="C25" s="1">
         <v>4.5</v>
       </c>
-      <c r="D25" s="1">
+      <c r="D25">
         <v>7</v>
       </c>
       <c r="E25">
@@ -1720,7 +1719,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="B26" t="s">
         <v>34</v>
@@ -1728,7 +1727,7 @@
       <c r="C26" s="1">
         <v>6.3999810000000004</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26">
         <v>11.5</v>
       </c>
       <c r="E26">
@@ -1745,7 +1744,7 @@
       <c r="C27" s="1">
         <v>2.5</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27">
         <v>6.5</v>
       </c>
       <c r="E27">
@@ -1762,7 +1761,7 @@
       <c r="C28" s="1">
         <v>2.75</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28">
         <v>4.5</v>
       </c>
       <c r="E28">
@@ -1771,7 +1770,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="B29" t="s">
         <v>39</v>
@@ -1779,7 +1778,7 @@
       <c r="C29" s="1">
         <v>1</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29">
         <v>3</v>
       </c>
       <c r="E29">
@@ -1793,7 +1792,7 @@
       <c r="B30" t="s">
         <v>41</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30">
         <v>5.5</v>
       </c>
       <c r="E30">
@@ -1810,7 +1809,7 @@
       <c r="C31" s="1">
         <v>16</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31">
         <v>27</v>
       </c>
       <c r="E31">
@@ -1827,7 +1826,7 @@
       <c r="C32" s="1">
         <v>9</v>
       </c>
-      <c r="D32" s="1">
+      <c r="D32">
         <v>15</v>
       </c>
       <c r="E32">
@@ -1844,7 +1843,7 @@
       <c r="C33" s="1">
         <v>5</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33">
         <v>10</v>
       </c>
       <c r="E33">
@@ -1861,7 +1860,7 @@
       <c r="C34" s="1">
         <v>4</v>
       </c>
-      <c r="D34" s="1">
+      <c r="D34">
         <v>10</v>
       </c>
       <c r="E34">
@@ -1878,7 +1877,7 @@
       <c r="C35" s="1">
         <v>3.25</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35">
         <v>6</v>
       </c>
       <c r="E35">
@@ -1895,7 +1894,7 @@
       <c r="C36" s="1">
         <v>6</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36">
         <v>10</v>
       </c>
       <c r="E36">
@@ -1912,7 +1911,7 @@
       <c r="C37" s="1">
         <v>4</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37">
         <v>6</v>
       </c>
       <c r="E37">
@@ -1929,7 +1928,7 @@
       <c r="C38" s="1">
         <v>3.25</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38">
         <v>5.5</v>
       </c>
       <c r="E38">
@@ -1946,7 +1945,7 @@
       <c r="C39" s="1">
         <v>2.5990000000000002</v>
       </c>
-      <c r="D39" s="1">
+      <c r="D39">
         <v>5</v>
       </c>
       <c r="E39">
@@ -1960,7 +1959,7 @@
       <c r="B40" t="s">
         <v>61</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40">
         <v>10</v>
       </c>
       <c r="E40">
@@ -1974,7 +1973,7 @@
       <c r="B41" t="s">
         <v>63</v>
       </c>
-      <c r="D41" s="1">
+      <c r="D41">
         <v>10</v>
       </c>
       <c r="E41">
@@ -1988,7 +1987,7 @@
       <c r="B42" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="1">
+      <c r="D42">
         <v>1.5</v>
       </c>
       <c r="E42">
@@ -2002,7 +2001,7 @@
       <c r="B43" t="s">
         <v>65</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43">
         <v>1.5</v>
       </c>
       <c r="E43">
@@ -2011,12 +2010,12 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="B44" t="s">
         <v>66</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44">
         <v>7</v>
       </c>
       <c r="E44">
@@ -2033,7 +2032,7 @@
       <c r="C45" s="1">
         <v>2.4</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45">
         <v>4</v>
       </c>
       <c r="E45">
@@ -2050,7 +2049,7 @@
       <c r="C46" s="1">
         <v>1.2656000000000001</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46">
         <v>4</v>
       </c>
       <c r="E46">
@@ -2067,7 +2066,7 @@
       <c r="C47" s="1">
         <v>1.72</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47">
         <v>4.5</v>
       </c>
       <c r="E47">
@@ -2084,7 +2083,7 @@
       <c r="C48" s="1">
         <v>2.12</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48">
         <v>4.5</v>
       </c>
       <c r="E48">
@@ -2101,7 +2100,7 @@
       <c r="C49" s="1">
         <v>43</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49">
         <v>60</v>
       </c>
       <c r="E49">
@@ -2118,7 +2117,7 @@
       <c r="C50" s="1">
         <v>33</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50">
         <v>55</v>
       </c>
       <c r="E50">
@@ -2132,7 +2131,7 @@
       <c r="B51" t="s">
         <v>80</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51">
         <v>40</v>
       </c>
       <c r="E51">
@@ -2149,7 +2148,7 @@
       <c r="C52" s="1">
         <v>3.75</v>
       </c>
-      <c r="D52" s="1">
+      <c r="D52">
         <v>6.5</v>
       </c>
       <c r="E52">
@@ -2166,7 +2165,7 @@
       <c r="C53" s="1">
         <v>80.998400000000004</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53">
         <v>96</v>
       </c>
       <c r="E53">
@@ -2183,7 +2182,7 @@
       <c r="C54" s="1">
         <v>11</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54">
         <v>17</v>
       </c>
       <c r="E54">
@@ -2194,7 +2193,7 @@
       <c r="B55" t="s">
         <v>86</v>
       </c>
-      <c r="D55" s="1">
+      <c r="D55">
         <v>24.5</v>
       </c>
       <c r="E55">
@@ -2208,7 +2207,7 @@
       <c r="B56" t="s">
         <v>88</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56">
         <v>67</v>
       </c>
       <c r="E56">
@@ -2222,7 +2221,7 @@
       <c r="B57" t="s">
         <v>90</v>
       </c>
-      <c r="D57" s="1">
+      <c r="D57">
         <v>52</v>
       </c>
       <c r="E57">
@@ -2239,7 +2238,7 @@
       <c r="C58" s="1">
         <v>35.499966999999998</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58">
         <v>55</v>
       </c>
       <c r="E58">
@@ -2253,7 +2252,7 @@
       <c r="B59" t="s">
         <v>92</v>
       </c>
-      <c r="D59" s="1">
+      <c r="D59">
         <v>5.5</v>
       </c>
       <c r="E59">
@@ -2270,7 +2269,7 @@
       <c r="C60" s="1">
         <v>7</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60">
         <v>11.5</v>
       </c>
       <c r="E60">
@@ -2284,7 +2283,7 @@
       <c r="B61" t="s">
         <v>96</v>
       </c>
-      <c r="D61" s="1">
+      <c r="D61">
         <v>11.5</v>
       </c>
       <c r="E61">
@@ -2301,7 +2300,7 @@
       <c r="C62" s="1">
         <v>7</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62">
         <v>11.5</v>
       </c>
       <c r="E62">
@@ -2318,7 +2317,7 @@
       <c r="C63" s="1">
         <v>23.500045</v>
       </c>
-      <c r="D63" s="1">
+      <c r="D63">
         <v>32</v>
       </c>
       <c r="E63">
@@ -2335,7 +2334,7 @@
       <c r="C64" s="1">
         <v>3.75</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64">
         <v>8</v>
       </c>
       <c r="E64">
@@ -2352,7 +2351,7 @@
       <c r="C65" s="1">
         <v>60</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65">
         <v>70</v>
       </c>
       <c r="E65">
@@ -2369,7 +2368,7 @@
       <c r="C66" s="1">
         <v>8</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66">
         <v>12</v>
       </c>
       <c r="E66">
@@ -2386,7 +2385,7 @@
       <c r="C67" s="1">
         <v>10</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67">
         <v>14.5</v>
       </c>
       <c r="E67">
@@ -2403,7 +2402,7 @@
       <c r="C68" s="1">
         <v>14</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68">
         <v>23</v>
       </c>
       <c r="E68">
@@ -2420,7 +2419,7 @@
       <c r="C69" s="1">
         <v>10.999985000000001</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69">
         <v>17.5</v>
       </c>
       <c r="E69">
@@ -2429,7 +2428,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B70" t="s">
         <v>113</v>
@@ -2437,7 +2436,7 @@
       <c r="C70" s="1">
         <v>10.531599999999999</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70">
         <v>20</v>
       </c>
       <c r="E70">
@@ -2454,7 +2453,7 @@
       <c r="C71" s="1">
         <v>0.4</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71">
         <v>1.5</v>
       </c>
       <c r="E71">
@@ -2471,7 +2470,7 @@
       <c r="C72" s="1">
         <v>1.1999470000000001</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72">
         <v>3</v>
       </c>
       <c r="E72">
@@ -2488,7 +2487,7 @@
       <c r="C73" s="1">
         <v>2</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73">
         <v>3.5</v>
       </c>
       <c r="E73">
@@ -2502,7 +2501,7 @@
       <c r="B74" t="s">
         <v>120</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74">
         <v>4</v>
       </c>
       <c r="E74">
@@ -2516,7 +2515,7 @@
       <c r="B75" t="s">
         <v>121</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75">
         <v>3</v>
       </c>
       <c r="E75">
@@ -2533,7 +2532,7 @@
       <c r="C76" s="1">
         <v>4</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76">
         <v>6.5</v>
       </c>
       <c r="E76">
@@ -2547,7 +2546,7 @@
       <c r="B77" t="s">
         <v>124</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77">
         <v>2</v>
       </c>
       <c r="E77">
@@ -2556,12 +2555,12 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="B78" t="s">
         <v>125</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78">
         <v>8</v>
       </c>
       <c r="E78">
@@ -2578,7 +2577,7 @@
       <c r="C79" s="1">
         <v>13</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79">
         <v>25</v>
       </c>
       <c r="E79">
@@ -2587,7 +2586,7 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="B80" t="s">
         <v>128</v>
@@ -2595,7 +2594,7 @@
       <c r="C80" s="1">
         <v>1.8999820000000001</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80">
         <v>5</v>
       </c>
       <c r="E80">
@@ -2612,7 +2611,7 @@
       <c r="C81" s="1">
         <v>3.75</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81">
         <v>7</v>
       </c>
       <c r="E81">
@@ -2621,7 +2620,7 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="B82" t="s">
         <v>131</v>
@@ -2629,7 +2628,7 @@
       <c r="C82" s="1">
         <v>0.38419999999999999</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82">
         <v>1</v>
       </c>
       <c r="E82">
@@ -2646,7 +2645,7 @@
       <c r="C83" s="1">
         <v>10</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83">
         <v>15</v>
       </c>
       <c r="E83">
@@ -2663,7 +2662,7 @@
       <c r="C84" s="1">
         <v>10</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84">
         <v>15</v>
       </c>
       <c r="E84">
@@ -2675,9 +2674,9 @@
         <v>761034</v>
       </c>
       <c r="B85" t="s">
-        <v>300</v>
-      </c>
-      <c r="D85" s="1">
+        <v>295</v>
+      </c>
+      <c r="D85">
         <v>0.25</v>
       </c>
       <c r="E85">
@@ -2694,7 +2693,7 @@
       <c r="C86" s="1">
         <v>9.3225000000000002E-2</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86">
         <v>0.25</v>
       </c>
       <c r="E86">
@@ -2711,7 +2710,7 @@
       <c r="C87" s="1">
         <v>9.3225000000000002E-2</v>
       </c>
-      <c r="D87" s="1">
+      <c r="D87">
         <v>0.25</v>
       </c>
       <c r="E87">
@@ -2728,7 +2727,7 @@
       <c r="C88" s="1">
         <v>0.5</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88">
         <v>1.5</v>
       </c>
       <c r="E88">
@@ -2745,7 +2744,7 @@
       <c r="C89" s="1">
         <v>15</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89">
         <v>20</v>
       </c>
       <c r="E89">
@@ -2762,7 +2761,7 @@
       <c r="C90" s="1">
         <v>7.9999479999999998</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90">
         <v>11</v>
       </c>
       <c r="E90">
@@ -2779,7 +2778,7 @@
       <c r="C91" s="1">
         <v>2.5</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91">
         <v>11</v>
       </c>
       <c r="E91">
@@ -2793,7 +2792,7 @@
       <c r="B92" t="s">
         <v>146</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92">
         <v>6</v>
       </c>
       <c r="E92">
@@ -2810,7 +2809,7 @@
       <c r="C93" s="1">
         <v>2.5</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93">
         <v>4</v>
       </c>
       <c r="E93">
@@ -2827,7 +2826,7 @@
       <c r="C94" s="1">
         <v>6.5</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94">
         <v>12</v>
       </c>
       <c r="E94">
@@ -2844,7 +2843,7 @@
       <c r="C95" s="1">
         <v>6.9494999999999996</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95">
         <v>12</v>
       </c>
       <c r="E95">
@@ -2861,7 +2860,7 @@
       <c r="C96" s="1">
         <v>12.5</v>
       </c>
-      <c r="D96" s="1">
+      <c r="D96">
         <v>17</v>
       </c>
       <c r="E96">
@@ -2878,7 +2877,7 @@
       <c r="C97" s="1">
         <v>0.90400000000000003</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97">
         <v>4</v>
       </c>
       <c r="E97">
@@ -2892,7 +2891,7 @@
       <c r="B98" t="s">
         <v>157</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98">
         <v>10</v>
       </c>
       <c r="E98">
@@ -2909,7 +2908,7 @@
       <c r="C99" s="1">
         <v>1</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99">
         <v>4.5</v>
       </c>
       <c r="E99">
@@ -2926,7 +2925,7 @@
       <c r="C100" s="1">
         <v>0.85</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100">
         <v>2</v>
       </c>
       <c r="E100">
@@ -2940,7 +2939,7 @@
       <c r="B101" t="s">
         <v>162</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101">
         <v>8</v>
       </c>
       <c r="E101">
@@ -2957,7 +2956,7 @@
       <c r="C102" s="1">
         <v>1.499962</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102">
         <v>3</v>
       </c>
       <c r="E102">
@@ -2974,7 +2973,7 @@
       <c r="C103" s="1">
         <v>7.9999479999999998</v>
       </c>
-      <c r="D103" s="1">
+      <c r="D103">
         <v>12</v>
       </c>
       <c r="E103">
@@ -2991,7 +2990,7 @@
       <c r="C104" s="1">
         <v>2.3165</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104">
         <v>5</v>
       </c>
       <c r="E104">
@@ -3002,7 +3001,7 @@
       <c r="B105" t="s">
         <v>167</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105">
         <v>6.5</v>
       </c>
       <c r="E105">
@@ -3013,7 +3012,7 @@
       <c r="B106" t="s">
         <v>168</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106">
         <v>8.5</v>
       </c>
       <c r="E106">
@@ -3022,7 +3021,7 @@
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="B107" t="s">
         <v>169</v>
@@ -3030,7 +3029,7 @@
       <c r="C107" s="1">
         <v>3.8420000000000001</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107">
         <v>6.5</v>
       </c>
       <c r="E107">
@@ -3047,7 +3046,7 @@
       <c r="C108" s="1">
         <v>5.7516999999999996</v>
       </c>
-      <c r="D108" s="1">
+      <c r="D108">
         <v>7.5</v>
       </c>
       <c r="E108">
@@ -3058,7 +3057,7 @@
       <c r="B109" t="s">
         <v>171</v>
       </c>
-      <c r="D109" s="1">
+      <c r="D109">
         <v>33</v>
       </c>
       <c r="E109">
@@ -3075,7 +3074,7 @@
       <c r="C110" s="1">
         <v>1.2543</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110">
         <v>3</v>
       </c>
       <c r="E110">
@@ -3089,7 +3088,7 @@
       <c r="B111" t="s">
         <v>175</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111">
         <v>3</v>
       </c>
       <c r="E111">
@@ -3106,7 +3105,7 @@
       <c r="C112" s="1">
         <v>4</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112">
         <v>12</v>
       </c>
       <c r="E112">
@@ -3117,7 +3116,7 @@
       <c r="B113" t="s">
         <v>178</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113">
         <v>85</v>
       </c>
       <c r="E113">
@@ -3134,7 +3133,7 @@
       <c r="C114" s="1">
         <v>12.999972</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114">
         <v>23</v>
       </c>
       <c r="E114">
@@ -3151,7 +3150,7 @@
       <c r="C115" s="1">
         <v>8.7010000000000004E-2</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115">
         <v>0.25</v>
       </c>
       <c r="E115">
@@ -3168,7 +3167,7 @@
       <c r="C116" s="1">
         <v>8.7010000000000004E-2</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116">
         <v>0.25</v>
       </c>
       <c r="E116">
@@ -3182,7 +3181,7 @@
       <c r="B117" t="s">
         <v>184</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117">
         <v>65</v>
       </c>
       <c r="E117">
@@ -3193,7 +3192,7 @@
       <c r="B118" t="s">
         <v>185</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118">
         <v>70</v>
       </c>
       <c r="E118">
@@ -3207,7 +3206,7 @@
       <c r="B119" t="s">
         <v>187</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119">
         <v>24</v>
       </c>
       <c r="E119">
@@ -3224,7 +3223,7 @@
       <c r="C120" s="1">
         <v>23</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120">
         <v>37</v>
       </c>
       <c r="E120">
@@ -3241,7 +3240,7 @@
       <c r="C121" s="1">
         <v>26.5</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121">
         <v>37</v>
       </c>
       <c r="E121">
@@ -3252,7 +3251,7 @@
       <c r="B122" t="s">
         <v>192</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122">
         <v>90</v>
       </c>
       <c r="E122">
@@ -3263,7 +3262,7 @@
       <c r="B123" t="s">
         <v>193</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123">
         <v>12</v>
       </c>
       <c r="E123">
@@ -3277,7 +3276,7 @@
       <c r="B124" t="s">
         <v>195</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124">
         <v>12</v>
       </c>
       <c r="E124">
@@ -3294,7 +3293,7 @@
       <c r="C125" s="1">
         <v>5.8872999999999998</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125">
         <v>12</v>
       </c>
       <c r="E125">
@@ -3311,7 +3310,7 @@
       <c r="C126" s="1">
         <v>5.7968999999999991</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126">
         <v>12</v>
       </c>
       <c r="E126">
@@ -3322,7 +3321,7 @@
       <c r="B127" t="s">
         <v>200</v>
       </c>
-      <c r="D127" s="1">
+      <c r="D127">
         <v>4</v>
       </c>
       <c r="E127">
@@ -3333,7 +3332,7 @@
       <c r="B128" t="s">
         <v>201</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128">
         <v>20</v>
       </c>
       <c r="E128">
@@ -3344,7 +3343,7 @@
       <c r="B129" t="s">
         <v>202</v>
       </c>
-      <c r="D129" s="1">
+      <c r="D129">
         <v>14.5</v>
       </c>
       <c r="E129">
@@ -3361,7 +3360,7 @@
       <c r="C130" s="1">
         <v>14.995100000000001</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130">
         <v>23</v>
       </c>
       <c r="E130">
@@ -3372,7 +3371,7 @@
       <c r="B131" t="s">
         <v>205</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131">
         <v>15</v>
       </c>
       <c r="E131">
@@ -3389,7 +3388,7 @@
       <c r="C132" s="1">
         <v>11</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132">
         <v>14.5</v>
       </c>
       <c r="E132">
@@ -3403,7 +3402,7 @@
       <c r="B133" t="s">
         <v>208</v>
       </c>
-      <c r="D133" s="1">
+      <c r="D133">
         <v>8</v>
       </c>
       <c r="E133">
@@ -3417,7 +3416,7 @@
       <c r="B134" t="s">
         <v>210</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134">
         <v>6</v>
       </c>
       <c r="E134">
@@ -3434,7 +3433,7 @@
       <c r="C135" s="1">
         <v>8</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135">
         <v>11</v>
       </c>
       <c r="E135">
@@ -3451,7 +3450,7 @@
       <c r="C136" s="1">
         <v>6.4999859999999998</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136">
         <v>8.5</v>
       </c>
       <c r="E136">
@@ -3462,7 +3461,7 @@
       <c r="B137" t="s">
         <v>214</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137">
         <v>45</v>
       </c>
       <c r="E137">
@@ -3479,7 +3478,7 @@
       <c r="C138" s="1">
         <v>16.79</v>
       </c>
-      <c r="D138" s="1">
+      <c r="D138">
         <v>28</v>
       </c>
       <c r="E138">
@@ -3493,7 +3492,7 @@
       <c r="B139" t="s">
         <v>217</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139">
         <v>35</v>
       </c>
       <c r="E139">
@@ -3507,7 +3506,7 @@
       <c r="B140" t="s">
         <v>218</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140">
         <v>35</v>
       </c>
       <c r="E140">
@@ -3524,7 +3523,7 @@
       <c r="C141" s="1">
         <v>12</v>
       </c>
-      <c r="D141" s="1">
+      <c r="D141">
         <v>18</v>
       </c>
       <c r="E141">
@@ -3541,7 +3540,7 @@
       <c r="C142" s="1">
         <v>12</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142">
         <v>18</v>
       </c>
       <c r="E142">
@@ -3558,7 +3557,7 @@
       <c r="C143" s="1">
         <v>1</v>
       </c>
-      <c r="D143" s="1">
+      <c r="D143">
         <v>3</v>
       </c>
       <c r="E143">
@@ -3570,12 +3569,12 @@
         <v>142</v>
       </c>
       <c r="B144" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="C144" s="1">
         <v>2</v>
       </c>
-      <c r="D144" s="1">
+      <c r="D144">
         <v>3.5</v>
       </c>
       <c r="E144">
@@ -3586,7 +3585,7 @@
       <c r="B145" t="s">
         <v>225</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145">
         <v>3.5</v>
       </c>
       <c r="E145">
@@ -3603,7 +3602,7 @@
       <c r="C146" s="1">
         <v>80.000045</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146">
         <v>97</v>
       </c>
       <c r="E146">
@@ -3620,7 +3619,7 @@
       <c r="C147" s="1">
         <v>18.5</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147">
         <v>23</v>
       </c>
       <c r="E147">
@@ -3634,7 +3633,7 @@
       <c r="B148" t="s">
         <v>231</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148">
         <v>30</v>
       </c>
       <c r="E148">
@@ -3648,7 +3647,7 @@
       <c r="B149" t="s">
         <v>233</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149">
         <v>10</v>
       </c>
       <c r="E149">
@@ -3665,7 +3664,7 @@
       <c r="C150" s="1">
         <v>0.75</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150">
         <v>3</v>
       </c>
       <c r="E150">
@@ -3682,7 +3681,7 @@
       <c r="C151" s="1">
         <v>1</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151">
         <v>2</v>
       </c>
       <c r="E151">
@@ -3699,7 +3698,7 @@
       <c r="C152" s="1">
         <v>18.500021</v>
       </c>
-      <c r="D152" s="1">
+      <c r="D152">
         <v>32.5</v>
       </c>
       <c r="E152">
@@ -3716,7 +3715,7 @@
       <c r="C153" s="1">
         <v>23.454844999999999</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153">
         <v>32.5</v>
       </c>
       <c r="E153">
@@ -3733,7 +3732,7 @@
       <c r="C154" s="1">
         <v>1.999987</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154">
         <v>4</v>
       </c>
       <c r="E154">
@@ -3744,7 +3743,7 @@
       <c r="B155" t="s">
         <v>242</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155">
         <v>8.5</v>
       </c>
       <c r="E155">
@@ -3755,7 +3754,7 @@
       <c r="B156" t="s">
         <v>243</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156">
         <v>7</v>
       </c>
       <c r="E156">
@@ -3772,7 +3771,7 @@
       <c r="C157" s="1">
         <v>1.25</v>
       </c>
-      <c r="D157" s="1">
+      <c r="D157">
         <v>4</v>
       </c>
       <c r="E157">
@@ -3783,7 +3782,7 @@
       <c r="B158" t="s">
         <v>246</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158">
         <v>4</v>
       </c>
       <c r="E158">
@@ -3800,7 +3799,7 @@
       <c r="C159" s="1">
         <v>15.499984</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159">
         <v>24</v>
       </c>
       <c r="E159">
@@ -3817,7 +3816,7 @@
       <c r="C160" s="1">
         <v>0.64410000000000001</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160">
         <v>1</v>
       </c>
       <c r="E160">
@@ -3831,7 +3830,7 @@
       <c r="B161" t="s">
         <v>251</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161">
         <v>6</v>
       </c>
       <c r="E161">
@@ -3848,7 +3847,7 @@
       <c r="C162" s="1">
         <v>7.5031999999999996</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162">
         <v>12</v>
       </c>
       <c r="E162">
@@ -3865,7 +3864,7 @@
       <c r="C163" s="1">
         <v>8.4862999999999982</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163">
         <v>13.5</v>
       </c>
       <c r="E163">
@@ -3876,7 +3875,7 @@
       <c r="B164" t="s">
         <v>256</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164">
         <v>12</v>
       </c>
       <c r="E164">
@@ -3893,7 +3892,7 @@
       <c r="C165" s="1">
         <v>8.904399999999999</v>
       </c>
-      <c r="D165" s="1">
+      <c r="D165">
         <v>13.5</v>
       </c>
       <c r="E165">
@@ -3907,7 +3906,7 @@
       <c r="B166" t="s">
         <v>260</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166">
         <v>10</v>
       </c>
       <c r="E166">
@@ -3924,7 +3923,7 @@
       <c r="C167" s="1">
         <v>3.5</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167">
         <v>6.5</v>
       </c>
       <c r="E167">
@@ -3941,7 +3940,7 @@
       <c r="C168" s="1">
         <v>2</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168">
         <v>6</v>
       </c>
       <c r="E168">
@@ -3958,7 +3957,7 @@
       <c r="C169" s="1">
         <v>0.85</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169">
         <v>3.5</v>
       </c>
       <c r="E169">
@@ -3975,7 +3974,7 @@
       <c r="C170" s="1">
         <v>21</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170">
         <v>24.5</v>
       </c>
       <c r="E170">
@@ -3992,7 +3991,7 @@
       <c r="C171" s="1">
         <v>16.500033999999999</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171">
         <v>23</v>
       </c>
       <c r="E171">
@@ -4004,12 +4003,12 @@
         <v>270</v>
       </c>
       <c r="B172" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C172" s="1">
         <v>5.5</v>
       </c>
-      <c r="D172" s="1">
+      <c r="D172">
         <v>9</v>
       </c>
       <c r="E172">
@@ -4026,7 +4025,7 @@
       <c r="C173" s="1">
         <v>2</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173">
         <v>6</v>
       </c>
       <c r="E173">
@@ -4037,7 +4036,7 @@
       <c r="B174" t="s">
         <v>273</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174">
         <v>1</v>
       </c>
       <c r="E174">
@@ -4051,7 +4050,7 @@
       <c r="B175" t="s">
         <v>274</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175">
         <v>4</v>
       </c>
       <c r="E175">
@@ -4062,7 +4061,7 @@
       <c r="B176" t="s">
         <v>275</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176">
         <v>4</v>
       </c>
       <c r="E176">
@@ -4079,7 +4078,7 @@
       <c r="C177" s="1">
         <v>2</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177">
         <v>5</v>
       </c>
       <c r="E177">
@@ -4096,7 +4095,7 @@
       <c r="C178" s="1">
         <v>2.75</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178">
         <v>6.5</v>
       </c>
       <c r="E178">
@@ -4113,7 +4112,7 @@
       <c r="C179" s="1">
         <v>2.75</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179">
         <v>6.5</v>
       </c>
       <c r="E179">
@@ -4127,7 +4126,7 @@
       <c r="B180" t="s">
         <v>281</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180">
         <v>6</v>
       </c>
       <c r="E180">
@@ -4141,7 +4140,7 @@
       <c r="B181" t="s">
         <v>282</v>
       </c>
-      <c r="D181" s="1">
+      <c r="D181">
         <v>2</v>
       </c>
       <c r="E181">
@@ -4152,7 +4151,7 @@
       <c r="B182" t="s">
         <v>283</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182">
         <v>50</v>
       </c>
       <c r="E182">

</xml_diff>